<commit_message>
Update Government Savings Automation Assessment with new metrics and documentation
- Revised the Executive Summary to include updated metrics and findings from the latest assessment.
- Added new CSV files for live validation registers, pipeline live validation, and endpoint current states for Mobile 1 and Mobile 2 APIs.
- Enhanced the technical assessment documentation to reflect the current state of automation coverage and CI integration.
- Updated the Government Savings Coverage Matrix and verified metrics register with the latest data.
- Improved the Render and Visual QA documentation to ensure accurate reporting of document exports.

These changes aim to provide a comprehensive overview of the automation coverage status and facilitate informed decision-making for future improvements.
</commit_message>
<xml_diff>
--- a/government-savings-automation-assessment/03-analysis/government-savings-coverage-matrix.xlsx
+++ b/government-savings-automation-assessment/03-analysis/government-savings-coverage-matrix.xlsx
@@ -61,17 +61,17 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FFE0B2"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
         <fgColor rgb="00ECEFF1"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00FFCDD2"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFE0B2"/>
       </patternFill>
     </fill>
   </fills>
@@ -87,7 +87,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -102,16 +102,13 @@
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment wrapText="1"/>
     </xf>
   </cellXfs>
@@ -479,7 +476,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G12"/>
+  <dimension ref="A1:G15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="48" customWidth="1" min="1" max="1"/>
@@ -487,7 +484,7 @@
     <col width="10" customWidth="1" min="3" max="3"/>
     <col width="11" customWidth="1" min="4" max="4"/>
     <col width="13" customWidth="1" min="5" max="5"/>
-    <col width="22" customWidth="1" min="6" max="6"/>
+    <col width="19" customWidth="1" min="6" max="6"/>
     <col width="17" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
@@ -546,27 +543,27 @@
     <row r="5">
       <c r="A5" s="3" t="inlineStr">
         <is>
-          <t>M-V3-UI</t>
+          <t>M-M2-IMPL</t>
         </is>
       </c>
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>V3 scoped TestNG nightly share</t>
+          <t>Mobile 2 business endpoint automation (code)</t>
         </is>
       </c>
       <c r="C5" s="3" t="inlineStr">
         <is>
-          <t>379/436</t>
+          <t>96.0%</t>
         </is>
       </c>
       <c r="D5" s="3" t="inlineStr">
         <is>
-          <t>379</t>
+          <t>24</t>
         </is>
       </c>
       <c r="E5" s="3" t="inlineStr">
         <is>
-          <t>436</t>
+          <t>25</t>
         </is>
       </c>
       <c r="F5" s="4" t="inlineStr">
@@ -583,69 +580,69 @@
     <row r="6">
       <c r="A6" s="3" t="inlineStr">
         <is>
-          <t>M-V2-UI</t>
+          <t>M-M2-EXEC</t>
         </is>
       </c>
       <c r="B6" s="3" t="inlineStr">
         <is>
-          <t>V2 UP-scoped qTest share</t>
+          <t>Mobile 2 last documented master run</t>
         </is>
       </c>
       <c r="C6" s="3" t="inlineStr">
         <is>
-          <t>268/744</t>
+          <t>88.0%</t>
         </is>
       </c>
       <c r="D6" s="3" t="inlineStr">
         <is>
-          <t>268</t>
+          <t>22</t>
         </is>
       </c>
       <c r="E6" s="3" t="inlineStr">
         <is>
-          <t>744</t>
-        </is>
-      </c>
-      <c r="F6" s="4" t="inlineStr">
-        <is>
-          <t>Verified</t>
+          <t>25</t>
+        </is>
+      </c>
+      <c r="F6" s="5" t="inlineStr">
+        <is>
+          <t>Stale</t>
         </is>
       </c>
       <c r="G6" s="3" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>Conditional</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="3" t="inlineStr">
         <is>
-          <t>M-M2-API-V</t>
+          <t>M-M2-CI</t>
         </is>
       </c>
       <c r="B7" s="3" t="inlineStr">
         <is>
-          <t>Mobile 2 verified endpoint automation</t>
+          <t>Mobile 2 GitLab scheduled job</t>
         </is>
       </c>
       <c r="C7" s="3" t="inlineStr">
         <is>
-          <t>22/25</t>
+          <t>0%</t>
         </is>
       </c>
       <c r="D7" s="3" t="inlineStr">
         <is>
-          <t>22</t>
+          <t>0</t>
         </is>
       </c>
       <c r="E7" s="3" t="inlineStr">
         <is>
-          <t>25</t>
+          <t>1</t>
         </is>
       </c>
       <c r="F7" s="4" t="inlineStr">
         <is>
-          <t>Verified</t>
+          <t>Verified gap</t>
         </is>
       </c>
       <c r="G7" s="3" t="inlineStr">
@@ -657,54 +654,54 @@
     <row r="8">
       <c r="A8" s="3" t="inlineStr">
         <is>
-          <t>M-M2-API-P</t>
+          <t>M-M1-IMPL</t>
         </is>
       </c>
       <c r="B8" s="3" t="inlineStr">
         <is>
-          <t>Mobile 2 code-implemented (pending sign-off)</t>
+          <t>Mobile 1 endpoint automation (code)</t>
         </is>
       </c>
       <c r="C8" s="3" t="inlineStr">
         <is>
-          <t>24/25</t>
+          <t>22.2%</t>
         </is>
       </c>
       <c r="D8" s="3" t="inlineStr">
         <is>
-          <t>24</t>
+          <t>6</t>
         </is>
       </c>
       <c r="E8" s="3" t="inlineStr">
         <is>
-          <t>25</t>
-        </is>
-      </c>
-      <c r="F8" s="5" t="inlineStr">
-        <is>
-          <t>Pending verification</t>
+          <t>27</t>
+        </is>
+      </c>
+      <c r="F8" s="4" t="inlineStr">
+        <is>
+          <t>Verified</t>
         </is>
       </c>
       <c r="G8" s="3" t="inlineStr">
         <is>
-          <t>Conditional</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="3" t="inlineStr">
         <is>
-          <t>M-M1-API-V</t>
+          <t>M-M1-EXEC</t>
         </is>
       </c>
       <c r="B9" s="3" t="inlineStr">
         <is>
-          <t>Mobile 1 verified endpoint automation</t>
+          <t>Mobile 1 execution-verified endpoints</t>
         </is>
       </c>
       <c r="C9" s="3" t="inlineStr">
         <is>
-          <t>1/27</t>
+          <t>3.7%</t>
         </is>
       </c>
       <c r="D9" s="3" t="inlineStr">
@@ -731,17 +728,17 @@
     <row r="10">
       <c r="A10" s="3" t="inlineStr">
         <is>
-          <t>M-M2-CI-D</t>
+          <t>M-M1-CI</t>
         </is>
       </c>
       <c r="B10" s="3" t="inlineStr">
         <is>
-          <t>Mobile 2 GitLab nightly integration</t>
+          <t>Mobile 1 GitLab scheduled job</t>
         </is>
       </c>
       <c r="C10" s="3" t="inlineStr">
         <is>
-          <t>0/1</t>
+          <t>0%</t>
         </is>
       </c>
       <c r="D10" s="3" t="inlineStr">
@@ -768,27 +765,27 @@
     <row r="11">
       <c r="A11" s="3" t="inlineStr">
         <is>
-          <t>M-V3-CI-E</t>
+          <t>M-V3-UI</t>
         </is>
       </c>
       <c r="B11" s="3" t="inlineStr">
         <is>
-          <t>V3 UI scheduled job hard-fail</t>
+          <t>V3 scoped TestNG nightly share</t>
         </is>
       </c>
       <c r="C11" s="3" t="inlineStr">
         <is>
-          <t>1/1</t>
+          <t>86.9%</t>
         </is>
       </c>
       <c r="D11" s="3" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>379</t>
         </is>
       </c>
       <c r="E11" s="3" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>436</t>
         </is>
       </c>
       <c r="F11" s="4" t="inlineStr">
@@ -805,35 +802,146 @@
     <row r="12">
       <c r="A12" s="3" t="inlineStr">
         <is>
+          <t>M-V2-UI</t>
+        </is>
+      </c>
+      <c r="B12" s="3" t="inlineStr">
+        <is>
+          <t>V2 UP-scoped qTest share</t>
+        </is>
+      </c>
+      <c r="C12" s="3" t="inlineStr">
+        <is>
+          <t>36.0%</t>
+        </is>
+      </c>
+      <c r="D12" s="3" t="inlineStr">
+        <is>
+          <t>268</t>
+        </is>
+      </c>
+      <c r="E12" s="3" t="inlineStr">
+        <is>
+          <t>744</t>
+        </is>
+      </c>
+      <c r="F12" s="5" t="inlineStr">
+        <is>
+          <t>Stale</t>
+        </is>
+      </c>
+      <c r="G12" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="3" t="inlineStr">
+        <is>
+          <t>M-V3-CI</t>
+        </is>
+      </c>
+      <c r="B13" s="3" t="inlineStr">
+        <is>
+          <t>V3 GitLab scheduled job</t>
+        </is>
+      </c>
+      <c r="C13" s="3" t="inlineStr">
+        <is>
+          <t>100%</t>
+        </is>
+      </c>
+      <c r="D13" s="3" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="E13" s="3" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="F13" s="4" t="inlineStr">
+        <is>
+          <t>Verified</t>
+        </is>
+      </c>
+      <c r="G13" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="3" t="inlineStr">
+        <is>
+          <t>M-META-CI</t>
+        </is>
+      </c>
+      <c r="B14" s="3" t="inlineStr">
+        <is>
+          <t>Metadataweb API GitLab job</t>
+        </is>
+      </c>
+      <c r="C14" s="3" t="inlineStr">
+        <is>
+          <t>100%</t>
+        </is>
+      </c>
+      <c r="D14" s="3" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="E14" s="3" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="F14" s="4" t="inlineStr">
+        <is>
+          <t>Verified</t>
+        </is>
+      </c>
+      <c r="G14" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="3" t="inlineStr">
+        <is>
           <t>M-GHA-M2</t>
         </is>
       </c>
-      <c r="B12" s="3" t="inlineStr">
-        <is>
-          <t>GitHub Actions Dashboard vertical slice</t>
-        </is>
-      </c>
-      <c r="C12" s="3" t="inlineStr">
-        <is>
-          <t>1/1</t>
-        </is>
-      </c>
-      <c r="D12" s="3" t="inlineStr">
+      <c r="B15" s="3" t="inlineStr">
+        <is>
+          <t>GHA Dashboard vertical slice</t>
+        </is>
+      </c>
+      <c r="C15" s="3" t="inlineStr">
+        <is>
+          <t>100%</t>
+        </is>
+      </c>
+      <c r="D15" s="3" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="E12" s="3" t="inlineStr">
+      <c r="E15" s="3" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="F12" s="6" t="inlineStr">
+      <c r="F15" s="5" t="inlineStr">
         <is>
           <t>Verified external</t>
         </is>
       </c>
-      <c r="G12" s="3" t="inlineStr">
+      <c r="G15" s="3" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
@@ -987,2140 +1095,2140 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="7" t="inlineStr">
+      <c r="A2" s="6" t="inlineStr">
         <is>
           <t>Universal Platform</t>
         </is>
       </c>
-      <c r="B2" s="7" t="inlineStr">
+      <c r="B2" s="6" t="inlineStr">
         <is>
           <t>V2 Unite UI</t>
         </is>
       </c>
-      <c r="C2" s="7" t="inlineStr">
+      <c r="C2" s="6" t="inlineStr">
         <is>
           <t>UI Cucumber TestNG</t>
         </is>
       </c>
-      <c r="D2" s="7" t="inlineStr">
+      <c r="D2" s="6" t="inlineStr">
         <is>
           <t>UP workstreams (Enrollment IDP ABLE Withdrawal)</t>
         </is>
       </c>
-      <c r="E2" s="7" t="inlineStr">
+      <c r="E2" s="6" t="inlineStr">
         <is>
           <t>unite-test-automation</t>
         </is>
       </c>
-      <c r="F2" s="7" t="inlineStr">
+      <c r="F2" s="6" t="inlineStr">
         <is>
           <t>Ant regression targets (stage1 daily weekly)</t>
         </is>
       </c>
-      <c r="G2" s="7" t="inlineStr">
+      <c r="G2" s="6" t="inlineStr">
         <is>
           <t>268 UP-scoped qTest cases mapped</t>
         </is>
       </c>
-      <c r="H2" s="7" t="inlineStr">
+      <c r="H2" s="6" t="inlineStr">
         <is>
           <t>744 executed qTest population</t>
         </is>
       </c>
-      <c r="I2" s="7" t="inlineStr">
+      <c r="I2" s="6" t="inlineStr">
         <is>
           <t>268</t>
         </is>
       </c>
-      <c r="J2" s="7" t="inlineStr">
+      <c r="J2" s="6" t="inlineStr">
         <is>
           <t>36.0% inventory share</t>
         </is>
       </c>
-      <c r="K2" s="7" t="inlineStr">
+      <c r="K2" s="6" t="inlineStr">
         <is>
           <t>Verified manually executable; Jenkins/Ant legacy</t>
         </is>
       </c>
-      <c r="L2" s="7" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="M2" s="7" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="N2" s="7" t="inlineStr">
+      <c r="L2" s="6" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="M2" s="6" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="N2" s="6" t="inlineStr">
         <is>
           <t>Referenced (UNITE-TB-REFRESH)</t>
         </is>
       </c>
-      <c r="O2" s="7" t="inlineStr">
+      <c r="O2" s="6" t="inlineStr">
         <is>
           <t>Soft gate / manual — schedule not verified in this pass</t>
         </is>
       </c>
-      <c r="P2" s="7" t="inlineStr">
+      <c r="P2" s="6" t="inlineStr">
         <is>
           <t>Both paths in suites</t>
         </is>
       </c>
-      <c r="Q2" s="7" t="inlineStr">
+      <c r="Q2" s="6" t="inlineStr">
         <is>
           <t>Stage1 Stage5 TB</t>
         </is>
       </c>
-      <c r="R2" s="7" t="inlineStr">
+      <c r="R2" s="6" t="inlineStr">
         <is>
           <t>universal-platform-coverage/01-analysis/10-reconciliation-ledger.md</t>
         </is>
       </c>
-      <c r="S2" s="7" t="inlineStr">
+      <c r="S2" s="6" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="T2" s="7" t="inlineStr">
+      <c r="T2" s="6" t="inlineStr">
         <is>
           <t>Verified recurring regression (legacy Jenkins)</t>
         </is>
       </c>
-      <c r="U2" s="7" t="inlineStr">
+      <c r="U2" s="6" t="inlineStr">
         <is>
           <t>Not requirement-level coverage; V2 total repo ~2176 scenarios / 1538 features</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="7" t="inlineStr">
+      <c r="A3" s="6" t="inlineStr">
         <is>
           <t>Universal Platform</t>
         </is>
       </c>
-      <c r="B3" s="7" t="inlineStr">
+      <c r="B3" s="6" t="inlineStr">
         <is>
           <t>V3 Unite UI</t>
         </is>
       </c>
-      <c r="C3" s="7" t="inlineStr">
+      <c r="C3" s="6" t="inlineStr">
         <is>
           <t>UI Cucumber TestNG</t>
         </is>
       </c>
-      <c r="D3" s="7" t="inlineStr">
+      <c r="D3" s="6" t="inlineStr">
         <is>
           <t>UP UE IDP Withdrawal (+ adjacent)</t>
         </is>
       </c>
-      <c r="E3" s="7" t="inlineStr">
+      <c r="E3" s="6" t="inlineStr">
         <is>
           <t>prime-test-automation</t>
         </is>
       </c>
-      <c r="F3" s="7" t="inlineStr">
+      <c r="F3" s="6" t="inlineStr">
         <is>
           <t>stage1-ue-regression-test + stage1-unite-regression-master</t>
         </is>
       </c>
-      <c r="G3" s="7" t="inlineStr">
+      <c r="G3" s="6" t="inlineStr">
         <is>
           <t>379 scoped TestNG methods</t>
         </is>
       </c>
-      <c r="H3" s="7" t="inlineStr">
+      <c r="H3" s="6" t="inlineStr">
         <is>
           <t>436 nightly TestNG population</t>
         </is>
       </c>
-      <c r="I3" s="7" t="inlineStr">
+      <c r="I3" s="6" t="inlineStr">
         <is>
           <t>379</t>
         </is>
       </c>
-      <c r="J3" s="7" t="inlineStr">
+      <c r="J3" s="6" t="inlineStr">
         <is>
           <t>86.9% inventory share</t>
         </is>
       </c>
-      <c r="K3" s="7" t="inlineStr">
+      <c r="K3" s="6" t="inlineStr">
         <is>
           <t>Verified recurring regression</t>
         </is>
       </c>
-      <c r="L3" s="7" t="inlineStr">
+      <c r="L3" s="6" t="inlineStr">
         <is>
           <t>scheduled_regression_job</t>
         </is>
       </c>
-      <c r="M3" s="7" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="N3" s="7" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="O3" s="7" t="inlineStr">
+      <c r="M3" s="6" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="N3" s="6" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="O3" s="6" t="inlineStr">
         <is>
           <t>Hard gate on scheduled job failure (exit 1)</t>
         </is>
       </c>
-      <c r="P3" s="7" t="inlineStr">
+      <c r="P3" s="6" t="inlineStr">
         <is>
           <t>IDP + non-IDP suites</t>
         </is>
       </c>
-      <c r="Q3" s="7" t="inlineStr">
+      <c r="Q3" s="6" t="inlineStr">
         <is>
           <t>Stage1 (scheduled)</t>
         </is>
       </c>
-      <c r="R3" s="7" t="inlineStr">
+      <c r="R3" s="6" t="inlineStr">
         <is>
           <t>prime-test-automation/.gitlab-ci.yml</t>
         </is>
       </c>
-      <c r="S3" s="7" t="inlineStr">
+      <c r="S3" s="6" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="T3" s="7" t="inlineStr">
+      <c r="T3" s="6" t="inlineStr">
         <is>
           <t>Verified recurring regression</t>
         </is>
       </c>
-      <c r="U3" s="7" t="inlineStr">
+      <c r="U3" s="6" t="inlineStr">
         <is>
           <t>Adjacent 57 methods (contributions CSR web reg) not in 379 subtotal</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="7" t="inlineStr">
+      <c r="A4" s="6" t="inlineStr">
         <is>
           <t>Universal Platform</t>
         </is>
       </c>
-      <c r="B4" s="7" t="inlineStr">
+      <c r="B4" s="6" t="inlineStr">
         <is>
           <t>V3 Unite UI</t>
         </is>
       </c>
-      <c r="C4" s="7" t="inlineStr">
+      <c r="C4" s="6" t="inlineStr">
         <is>
           <t>UI Cucumber</t>
         </is>
       </c>
-      <c r="D4" s="7" t="inlineStr">
+      <c r="D4" s="6" t="inlineStr">
         <is>
           <t>Entity platform adjacent</t>
         </is>
       </c>
-      <c r="E4" s="7" t="inlineStr">
+      <c r="E4" s="6" t="inlineStr">
         <is>
           <t>prime-test-automation</t>
         </is>
       </c>
-      <c r="F4" s="7" t="inlineStr">
+      <c r="F4" s="6" t="inlineStr">
         <is>
           <t>unite-entity module</t>
         </is>
       </c>
-      <c r="G4" s="7" t="inlineStr">
+      <c r="G4" s="6" t="inlineStr">
         <is>
           <t>6 scenarios</t>
         </is>
       </c>
-      <c r="H4" s="7" t="inlineStr">
+      <c r="H4" s="6" t="inlineStr">
         <is>
           <t>TBD business denominator</t>
         </is>
       </c>
-      <c r="I4" s="7" t="inlineStr">
+      <c r="I4" s="6" t="inlineStr">
         <is>
           <t>6</t>
         </is>
       </c>
-      <c r="J4" s="7" t="inlineStr">
+      <c r="J4" s="6" t="inlineStr">
         <is>
           <t>TBD</t>
         </is>
       </c>
-      <c r="K4" s="7" t="inlineStr">
+      <c r="K4" s="6" t="inlineStr">
         <is>
           <t>Module suite in repo</t>
         </is>
       </c>
-      <c r="L4" s="7" t="inlineStr">
+      <c r="L4" s="6" t="inlineStr">
         <is>
           <t>Partial (same nightly job may not include entity)</t>
         </is>
       </c>
-      <c r="M4" s="7" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="N4" s="7" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="O4" s="7" t="inlineStr">
+      <c r="M4" s="6" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="N4" s="6" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="O4" s="6" t="inlineStr">
         <is>
           <t>Unknown</t>
         </is>
       </c>
-      <c r="P4" s="7" t="inlineStr">
+      <c r="P4" s="6" t="inlineStr">
         <is>
           <t>TBD</t>
         </is>
       </c>
-      <c r="Q4" s="7" t="inlineStr">
+      <c r="Q4" s="6" t="inlineStr">
         <is>
           <t>Stage1</t>
         </is>
       </c>
-      <c r="R4" s="7" t="inlineStr">
+      <c r="R4" s="6" t="inlineStr">
         <is>
           <t>prime-test-automation/unite/unite-entity/</t>
         </is>
       </c>
-      <c r="S4" s="7" t="inlineStr">
+      <c r="S4" s="6" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="T4" s="7" t="inlineStr">
+      <c r="T4" s="6" t="inlineStr">
         <is>
           <t>Verified manually executable</t>
         </is>
       </c>
-      <c r="U4" s="7" t="inlineStr">
+      <c r="U4" s="6" t="inlineStr">
         <is>
           <t>Pipeline inclusion for entity module not confirmed</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="7" t="inlineStr">
+      <c r="A5" s="6" t="inlineStr">
         <is>
           <t>Traditional Unite</t>
         </is>
       </c>
-      <c r="B5" s="7" t="inlineStr">
+      <c r="B5" s="6" t="inlineStr">
         <is>
           <t>V2 UI full surface</t>
         </is>
       </c>
-      <c r="C5" s="7" t="inlineStr">
+      <c r="C5" s="6" t="inlineStr">
         <is>
           <t>UI Cucumber</t>
         </is>
       </c>
-      <c r="D5" s="7" t="inlineStr">
+      <c r="D5" s="6" t="inlineStr">
         <is>
           <t>All V2 frontoffice + backoffice</t>
         </is>
       </c>
-      <c r="E5" s="7" t="inlineStr">
+      <c r="E5" s="6" t="inlineStr">
         <is>
           <t>unite-test-automation</t>
         </is>
       </c>
-      <c r="F5" s="7" t="inlineStr">
+      <c r="F5" s="6" t="inlineStr">
         <is>
           <t>Full testsuite tree</t>
         </is>
       </c>
-      <c r="G5" s="7" t="inlineStr">
+      <c r="G5" s="6" t="inlineStr">
         <is>
           <t>2176 scenarios (feature scan)</t>
         </is>
       </c>
-      <c r="H5" s="7" t="inlineStr">
+      <c r="H5" s="6" t="inlineStr">
         <is>
           <t>TBD approved business scope</t>
         </is>
       </c>
-      <c r="I5" s="7" t="inlineStr">
+      <c r="I5" s="6" t="inlineStr">
         <is>
           <t>TBD</t>
         </is>
       </c>
-      <c r="J5" s="7" t="inlineStr">
+      <c r="J5" s="6" t="inlineStr">
         <is>
           <t>TBD</t>
         </is>
       </c>
-      <c r="K5" s="7" t="inlineStr">
+      <c r="K5" s="6" t="inlineStr">
         <is>
           <t>Verified manually executable</t>
         </is>
       </c>
-      <c r="L5" s="7" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="M5" s="7" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="N5" s="7" t="inlineStr">
+      <c r="L5" s="6" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="M5" s="6" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="N5" s="6" t="inlineStr">
         <is>
           <t>Jenkins Ant targets</t>
         </is>
       </c>
-      <c r="O5" s="7" t="inlineStr">
+      <c r="O5" s="6" t="inlineStr">
         <is>
           <t>Manual / soft</t>
         </is>
       </c>
-      <c r="P5" s="7" t="inlineStr">
+      <c r="P5" s="6" t="inlineStr">
         <is>
           <t>Both</t>
         </is>
       </c>
-      <c r="Q5" s="7" t="inlineStr">
+      <c r="Q5" s="6" t="inlineStr">
         <is>
           <t>Stage1 Stage5</t>
         </is>
       </c>
-      <c r="R5" s="7" t="inlineStr">
+      <c r="R5" s="6" t="inlineStr">
         <is>
           <t>unite/testsuite/ (1538 features)</t>
         </is>
       </c>
-      <c r="S5" s="7" t="inlineStr">
+      <c r="S5" s="6" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="T5" s="7" t="inlineStr">
+      <c r="T5" s="6" t="inlineStr">
         <is>
           <t>Verified manually executable</t>
         </is>
       </c>
-      <c r="U5" s="7" t="inlineStr">
+      <c r="U5" s="6" t="inlineStr">
         <is>
           <t>Backoffice 1077 scenarios — not all in nightly subset</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="7" t="inlineStr">
+      <c r="A6" s="6" t="inlineStr">
         <is>
           <t>Traditional Unite</t>
         </is>
       </c>
-      <c r="B6" s="7" t="inlineStr">
+      <c r="B6" s="6" t="inlineStr">
         <is>
           <t>V2 Backoffice</t>
         </is>
       </c>
-      <c r="C6" s="7" t="inlineStr">
+      <c r="C6" s="6" t="inlineStr">
         <is>
           <t>UI Cucumber</t>
         </is>
       </c>
-      <c r="D6" s="7" t="inlineStr">
+      <c r="D6" s="6" t="inlineStr">
         <is>
           <t>Backoffice batch feeds Kofax</t>
         </is>
       </c>
-      <c r="E6" s="7" t="inlineStr">
+      <c r="E6" s="6" t="inlineStr">
         <is>
           <t>unite-test-automation</t>
         </is>
       </c>
-      <c r="F6" s="7" t="inlineStr">
+      <c r="F6" s="6" t="inlineStr">
         <is>
           <t>regression-backoffice-daily</t>
         </is>
       </c>
-      <c r="G6" s="7" t="inlineStr">
+      <c r="G6" s="6" t="inlineStr">
         <is>
           <t>1077 scenarios (backoffice subtree)</t>
         </is>
       </c>
-      <c r="H6" s="7" t="inlineStr">
+      <c r="H6" s="6" t="inlineStr">
         <is>
           <t>TBD</t>
         </is>
       </c>
-      <c r="I6" s="7" t="inlineStr">
+      <c r="I6" s="6" t="inlineStr">
         <is>
           <t>1077</t>
         </is>
       </c>
-      <c r="J6" s="7" t="inlineStr">
+      <c r="J6" s="6" t="inlineStr">
         <is>
           <t>TBD</t>
         </is>
       </c>
-      <c r="K6" s="7" t="inlineStr">
+      <c r="K6" s="6" t="inlineStr">
         <is>
           <t>Verified manually executable</t>
         </is>
       </c>
-      <c r="L6" s="7" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="M6" s="7" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="N6" s="7" t="inlineStr">
+      <c r="L6" s="6" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="M6" s="6" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="N6" s="6" t="inlineStr">
         <is>
           <t>Jenkins</t>
         </is>
       </c>
-      <c r="O6" s="7" t="inlineStr">
+      <c r="O6" s="6" t="inlineStr">
         <is>
           <t>Manual</t>
         </is>
       </c>
-      <c r="P6" s="7" t="inlineStr">
+      <c r="P6" s="6" t="inlineStr">
         <is>
           <t>Non-IDP typical</t>
         </is>
       </c>
-      <c r="Q6" s="7" t="inlineStr">
+      <c r="Q6" s="6" t="inlineStr">
         <is>
           <t>Stage1</t>
         </is>
       </c>
-      <c r="R6" s="7" t="inlineStr">
+      <c r="R6" s="6" t="inlineStr">
         <is>
           <t>unite/bin/build.xml + testsuite/backoffice/</t>
         </is>
       </c>
-      <c r="S6" s="7" t="inlineStr">
+      <c r="S6" s="6" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="T6" s="7" t="inlineStr">
+      <c r="T6" s="6" t="inlineStr">
         <is>
           <t>Verified manually executable</t>
         </is>
       </c>
-      <c r="U6" s="7" t="inlineStr">
+      <c r="U6" s="6" t="inlineStr">
         <is>
           <t>Not confirmed in GitLab nightly; separate from V3 schedule</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="7" t="inlineStr">
+      <c r="A7" s="6" t="inlineStr">
         <is>
           <t>ASTRO SFRP</t>
         </is>
       </c>
-      <c r="B7" s="7" t="inlineStr">
+      <c r="B7" s="6" t="inlineStr">
         <is>
           <t>ASTRO UI</t>
         </is>
       </c>
-      <c r="C7" s="7" t="inlineStr">
+      <c r="C7" s="6" t="inlineStr">
         <is>
           <t>UI Cucumber</t>
         </is>
       </c>
-      <c r="D7" s="7" t="inlineStr">
+      <c r="D7" s="6" t="inlineStr">
         <is>
           <t>ORS CAS ILS backoffice</t>
         </is>
       </c>
-      <c r="E7" s="7" t="inlineStr">
+      <c r="E7" s="6" t="inlineStr">
         <is>
           <t>astro-test-automation</t>
         </is>
       </c>
-      <c r="F7" s="7" t="inlineStr">
+      <c r="F7" s="6" t="inlineStr">
         <is>
           <t>Ant regression + daily testbed</t>
         </is>
       </c>
-      <c r="G7" s="7" t="inlineStr">
+      <c r="G7" s="6" t="inlineStr">
         <is>
           <t>1236 scenarios (391 features)</t>
         </is>
       </c>
-      <c r="H7" s="7" t="inlineStr">
+      <c r="H7" s="6" t="inlineStr">
         <is>
           <t>TBD approved scope</t>
         </is>
       </c>
-      <c r="I7" s="7" t="inlineStr">
+      <c r="I7" s="6" t="inlineStr">
         <is>
           <t>TBD</t>
         </is>
       </c>
-      <c r="J7" s="7" t="inlineStr">
+      <c r="J7" s="6" t="inlineStr">
         <is>
           <t>TBD</t>
         </is>
       </c>
-      <c r="K7" s="7" t="inlineStr">
+      <c r="K7" s="6" t="inlineStr">
         <is>
           <t>Verified manually executable</t>
         </is>
       </c>
-      <c r="L7" s="7" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="M7" s="7" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="N7" s="7" t="inlineStr">
+      <c r="L7" s="6" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="M7" s="6" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="N7" s="6" t="inlineStr">
         <is>
           <t>ASTRO-TB-REFRESH</t>
         </is>
       </c>
-      <c r="O7" s="7" t="inlineStr">
+      <c r="O7" s="6" t="inlineStr">
         <is>
           <t>Manual</t>
         </is>
       </c>
-      <c r="P7" s="7" t="inlineStr">
+      <c r="P7" s="6" t="inlineStr">
         <is>
           <t>Both</t>
         </is>
       </c>
-      <c r="Q7" s="7" t="inlineStr">
+      <c r="Q7" s="6" t="inlineStr">
         <is>
           <t>TB1 Stage1</t>
         </is>
       </c>
-      <c r="R7" s="7" t="inlineStr">
+      <c r="R7" s="6" t="inlineStr">
         <is>
           <t>astro/bin/build.xml</t>
         </is>
       </c>
-      <c r="S7" s="7" t="inlineStr">
+      <c r="S7" s="6" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="T7" s="7" t="inlineStr">
+      <c r="T7" s="6" t="inlineStr">
         <is>
           <t>Automation exists — schedule unverified</t>
         </is>
       </c>
-      <c r="U7" s="7" t="inlineStr">
+      <c r="U7" s="6" t="inlineStr">
         <is>
           <t>Not part of V2/V3 GitLab nightly</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="7" t="inlineStr">
+      <c r="A8" s="6" t="inlineStr">
         <is>
           <t>Unite MSC</t>
         </is>
       </c>
-      <c r="B8" s="7" t="inlineStr">
+      <c r="B8" s="6" t="inlineStr">
         <is>
           <t>Mobile 2 API</t>
         </is>
       </c>
-      <c r="C8" s="7" t="inlineStr">
+      <c r="C8" s="6" t="inlineStr">
         <is>
           <t>API TestNG RestAssured</t>
         </is>
       </c>
-      <c r="D8" s="7" t="inlineStr">
+      <c r="D8" s="6" t="inlineStr">
         <is>
           <t>MSC BFF business endpoints</t>
         </is>
       </c>
-      <c r="E8" s="7" t="inlineStr">
+      <c r="E8" s="6" t="inlineStr">
         <is>
           <t>api-test-automation</t>
         </is>
       </c>
-      <c r="F8" s="7" t="inlineStr">
+      <c r="F8" s="6" t="inlineStr">
         <is>
           <t>mobile-ms-master-regression</t>
         </is>
       </c>
-      <c r="G8" s="7" t="inlineStr">
+      <c r="G8" s="6" t="inlineStr">
         <is>
           <t>22 verified L3+ endpoints</t>
         </is>
       </c>
-      <c r="H8" s="7" t="inlineStr">
+      <c r="H8" s="6" t="inlineStr">
         <is>
           <t>25 documented business endpoints</t>
         </is>
       </c>
-      <c r="I8" s="7" t="inlineStr">
+      <c r="I8" s="6" t="inlineStr">
         <is>
           <t>22</t>
         </is>
       </c>
-      <c r="J8" s="7" t="inlineStr">
+      <c r="J8" s="6" t="inlineStr">
         <is>
           <t>88.0% verified endpoint automation</t>
         </is>
       </c>
-      <c r="K8" s="7" t="inlineStr">
+      <c r="K8" s="6" t="inlineStr">
         <is>
           <t>Verified sign-off 2026-07-14; projected 24/25 (96%) pending QC4+Stage1 rerun</t>
         </is>
       </c>
-      <c r="L8" s="7" t="inlineStr">
+      <c r="L8" s="6" t="inlineStr">
         <is>
           <t>No scheduled mobile job</t>
         </is>
       </c>
-      <c r="M8" s="7" t="inlineStr">
+      <c r="M8" s="6" t="inlineStr">
         <is>
           <t>GHA Dashboard slice validated external; module expansion in progress</t>
         </is>
       </c>
-      <c r="N8" s="7" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="O8" s="7" t="inlineStr">
+      <c r="N8" s="6" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="O8" s="6" t="inlineStr">
         <is>
           <t>No gate yet</t>
         </is>
       </c>
-      <c r="P8" s="7" t="inlineStr">
+      <c r="P8" s="6" t="inlineStr">
         <is>
           <t>okdirect + nmdirect</t>
         </is>
       </c>
-      <c r="Q8" s="7" t="inlineStr">
+      <c r="Q8" s="6" t="inlineStr">
         <is>
           <t>QC4 Stage1</t>
         </is>
       </c>
-      <c r="R8" s="7" t="inlineStr">
+      <c r="R8" s="6" t="inlineStr">
         <is>
           <t>17-mobile2-api-automation-signoff.md @ 7ccaf46; code @ cee0de9</t>
         </is>
       </c>
-      <c r="S8" s="7" t="inlineStr">
+      <c r="S8" s="6" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="T8" s="7" t="inlineStr">
+      <c r="T8" s="6" t="inlineStr">
         <is>
           <t>Verified baseline — sign-off path open</t>
         </is>
       </c>
-      <c r="U8" s="7" t="inlineStr">
+      <c r="U8" s="6" t="inlineStr">
         <is>
           <t>YTD + GET mobilebanks/{id} in code pending evidence; mobilemembers excluded from automation numerator; QA-1405 nightly</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="7" t="inlineStr">
+      <c r="A9" s="6" t="inlineStr">
         <is>
           <t>Unite MSC</t>
         </is>
       </c>
-      <c r="B9" s="7" t="inlineStr">
+      <c r="B9" s="6" t="inlineStr">
         <is>
           <t>Mobile 1 API</t>
         </is>
       </c>
-      <c r="C9" s="7" t="inlineStr">
+      <c r="C9" s="6" t="inlineStr">
         <is>
           <t>API TestNG RestAssured</t>
         </is>
       </c>
-      <c r="D9" s="7" t="inlineStr">
+      <c r="D9" s="6" t="inlineStr">
         <is>
           <t>MSC member session profile owner beneficiary bank</t>
         </is>
       </c>
-      <c r="E9" s="7" t="inlineStr">
+      <c r="E9" s="6" t="inlineStr">
         <is>
           <t>api-test-automation</t>
         </is>
       </c>
-      <c r="F9" s="7" t="inlineStr">
+      <c r="F9" s="6" t="inlineStr">
         <is>
           <t>mobile1-* profiles</t>
         </is>
       </c>
-      <c r="G9" s="7" t="inlineStr">
+      <c r="G9" s="6" t="inlineStr">
         <is>
           <t>1 verified + 5 implemented pending</t>
         </is>
       </c>
-      <c r="H9" s="7" t="inlineStr">
+      <c r="H9" s="6" t="inlineStr">
         <is>
           <t>27 documented business endpoints</t>
         </is>
       </c>
-      <c r="I9" s="7" t="inlineStr">
+      <c r="I9" s="6" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="J9" s="7" t="inlineStr">
+      <c r="J9" s="6" t="inlineStr">
         <is>
           <t>3.7% verified (1/27)</t>
         </is>
       </c>
-      <c r="K9" s="7" t="inlineStr">
+      <c r="K9" s="6" t="inlineStr">
         <is>
           <t>Verified session; 5 endpoints implemented pending evidence</t>
         </is>
       </c>
-      <c r="L9" s="7" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="M9" s="7" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="N9" s="7" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="O9" s="7" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="P9" s="7" t="inlineStr">
+      <c r="L9" s="6" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="M9" s="6" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="N9" s="6" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="O9" s="6" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="P9" s="6" t="inlineStr">
         <is>
           <t>okdirect + nmdirect (auth)</t>
         </is>
       </c>
-      <c r="Q9" s="7" t="inlineStr">
+      <c r="Q9" s="6" t="inlineStr">
         <is>
           <t>QC4 Stage1</t>
         </is>
       </c>
-      <c r="R9" s="7" t="inlineStr">
+      <c r="R9" s="6" t="inlineStr">
         <is>
           <t>03-document-postman-coverage-matrix.md; mobile/mobile1 @ cee0de9</t>
         </is>
       </c>
-      <c r="S9" s="7" t="inlineStr">
+      <c r="S9" s="6" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="T9" s="7" t="inlineStr">
+      <c r="T9" s="6" t="inlineStr">
         <is>
           <t>In progress — sprint 26.11</t>
         </is>
       </c>
-      <c r="U9" s="7" t="inlineStr">
+      <c r="U9" s="6" t="inlineStr">
         <is>
           <t>Leadership baseline 1/27; potential 6/27 after workbook mapping + execution evidence</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="7" t="inlineStr">
+      <c r="A10" s="6" t="inlineStr">
         <is>
           <t>Unite MSC</t>
         </is>
       </c>
-      <c r="B10" s="7" t="inlineStr">
+      <c r="B10" s="6" t="inlineStr">
         <is>
           <t>Mobile enrollment API</t>
         </is>
       </c>
-      <c r="C10" s="7" t="inlineStr">
+      <c r="C10" s="6" t="inlineStr">
         <is>
           <t>API TestNG</t>
         </is>
       </c>
-      <c r="D10" s="7" t="inlineStr">
+      <c r="D10" s="6" t="inlineStr">
         <is>
           <t>bootstrap smoke regression</t>
         </is>
       </c>
-      <c r="E10" s="7" t="inlineStr">
+      <c r="E10" s="6" t="inlineStr">
         <is>
           <t>api-test-automation</t>
         </is>
       </c>
-      <c r="F10" s="7" t="inlineStr">
+      <c r="F10" s="6" t="inlineStr">
         <is>
           <t>mobile-ms-bootstrap smoke regression</t>
         </is>
       </c>
-      <c r="G10" s="7" t="inlineStr">
+      <c r="G10" s="6" t="inlineStr">
         <is>
           <t>1 bootstrap class + suites</t>
         </is>
       </c>
-      <c r="H10" s="7" t="inlineStr">
+      <c r="H10" s="6" t="inlineStr">
         <is>
           <t>TBD enrollment scope</t>
         </is>
       </c>
-      <c r="I10" s="7" t="inlineStr">
+      <c r="I10" s="6" t="inlineStr">
         <is>
           <t>TBD</t>
         </is>
       </c>
-      <c r="J10" s="7" t="inlineStr">
+      <c r="J10" s="6" t="inlineStr">
         <is>
           <t>TBD</t>
         </is>
       </c>
-      <c r="K10" s="7" t="inlineStr">
+      <c r="K10" s="6" t="inlineStr">
         <is>
           <t>Verified manually executable</t>
         </is>
       </c>
-      <c r="L10" s="7" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="M10" s="7" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="N10" s="7" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="O10" s="7" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="P10" s="7" t="inlineStr">
+      <c r="L10" s="6" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="M10" s="6" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="N10" s="6" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="O10" s="6" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="P10" s="6" t="inlineStr">
         <is>
           <t>TBD</t>
         </is>
       </c>
-      <c r="Q10" s="7" t="inlineStr">
+      <c r="Q10" s="6" t="inlineStr">
         <is>
           <t>QC4 Stage1</t>
         </is>
       </c>
-      <c r="R10" s="7" t="inlineStr">
+      <c r="R10" s="6" t="inlineStr">
         <is>
           <t>mobile/enrollment/</t>
         </is>
       </c>
-      <c r="S10" s="7" t="inlineStr">
+      <c r="S10" s="6" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="T10" s="7" t="inlineStr">
+      <c r="T10" s="6" t="inlineStr">
         <is>
           <t>Verified manually executable</t>
         </is>
       </c>
-      <c r="U10" s="7" t="inlineStr">
+      <c r="U10" s="6" t="inlineStr">
         <is>
           <t>Small footprint; not nightly scheduled</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="7" t="inlineStr">
+      <c r="A11" s="6" t="inlineStr">
         <is>
           <t>Universal Platform</t>
         </is>
       </c>
-      <c r="B11" s="7" t="inlineStr">
+      <c r="B11" s="6" t="inlineStr">
         <is>
           <t>JSON API metadata</t>
         </is>
       </c>
-      <c r="C11" s="7" t="inlineStr">
+      <c r="C11" s="6" t="inlineStr">
         <is>
           <t>API TestNG</t>
         </is>
       </c>
-      <c r="D11" s="7" t="inlineStr">
+      <c r="D11" s="6" t="inlineStr">
         <is>
           <t>metadata web services</t>
         </is>
       </c>
-      <c r="E11" s="7" t="inlineStr">
+      <c r="E11" s="6" t="inlineStr">
         <is>
           <t>api-test-automation</t>
         </is>
       </c>
-      <c r="F11" s="7" t="inlineStr">
+      <c r="F11" s="6" t="inlineStr">
         <is>
           <t>stage1-api-metadata-pipeline</t>
         </is>
       </c>
-      <c r="G11" s="7" t="inlineStr">
+      <c r="G11" s="6" t="inlineStr">
         <is>
           <t>TestNG suite</t>
         </is>
       </c>
-      <c r="H11" s="7" t="inlineStr">
+      <c r="H11" s="6" t="inlineStr">
         <is>
           <t>~269 methods in universal modules (excluded from UP headline)</t>
         </is>
       </c>
-      <c r="I11" s="7" t="inlineStr">
+      <c r="I11" s="6" t="inlineStr">
         <is>
           <t>11 UP-scoped ops per UP assessment</t>
         </is>
       </c>
-      <c r="J11" s="7" t="inlineStr">
+      <c r="J11" s="6" t="inlineStr">
         <is>
           <t>11</t>
         </is>
       </c>
-      <c r="K11" s="7" t="inlineStr">
+      <c r="K11" s="6" t="inlineStr">
         <is>
           <t>TBD operation-level</t>
         </is>
       </c>
-      <c r="L11" s="7" t="inlineStr">
+      <c r="L11" s="6" t="inlineStr">
         <is>
           <t>Verified recurring regression</t>
         </is>
       </c>
-      <c r="M11" s="7" t="inlineStr">
+      <c r="M11" s="6" t="inlineStr">
         <is>
           <t>scheduled_metadataweb_stage1</t>
         </is>
       </c>
-      <c r="N11" s="7" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="O11" s="7" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="P11" s="7" t="inlineStr">
+      <c r="N11" s="6" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="O11" s="6" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="P11" s="6" t="inlineStr">
         <is>
           <t>Hard gate on job failure</t>
         </is>
       </c>
-      <c r="Q11" s="7" t="inlineStr">
+      <c r="Q11" s="6" t="inlineStr">
         <is>
           <t>TBD</t>
         </is>
       </c>
-      <c r="R11" s="7" t="inlineStr">
+      <c r="R11" s="6" t="inlineStr">
         <is>
           <t>Stage1</t>
         </is>
       </c>
-      <c r="S11" s="7" t="inlineStr">
+      <c r="S11" s="6" t="inlineStr">
         <is>
           <t>api-test-automation/.gitlab-ci.yml</t>
         </is>
       </c>
-      <c r="T11" s="7" t="inlineStr">
+      <c r="T11" s="6" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="U11" s="7" t="inlineStr">
+      <c r="U11" s="6" t="inlineStr">
         <is>
           <t>Verified recurring regression</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="7" t="inlineStr">
+      <c r="A12" s="6" t="inlineStr">
         <is>
           <t>Universal Platform</t>
         </is>
       </c>
-      <c r="B12" s="7" t="inlineStr">
+      <c r="B12" s="6" t="inlineStr">
         <is>
           <t>JSON API (account auth financial risk)</t>
         </is>
       </c>
-      <c r="C12" s="7" t="inlineStr">
+      <c r="C12" s="6" t="inlineStr">
         <is>
           <t>API TestNG</t>
         </is>
       </c>
-      <c r="D12" s="7" t="inlineStr">
+      <c r="D12" s="6" t="inlineStr">
         <is>
           <t>UP microservice APIs</t>
         </is>
       </c>
-      <c r="E12" s="7" t="inlineStr">
+      <c r="E12" s="6" t="inlineStr">
         <is>
           <t>api-test-automation</t>
         </is>
       </c>
-      <c r="F12" s="7" t="inlineStr">
+      <c r="F12" s="6" t="inlineStr">
         <is>
           <t>Per-module testng.xml</t>
         </is>
       </c>
-      <c r="G12" s="7" t="inlineStr">
+      <c r="G12" s="6" t="inlineStr">
         <is>
           <t>38 test classes universal/</t>
         </is>
       </c>
-      <c r="H12" s="7" t="inlineStr">
+      <c r="H12" s="6" t="inlineStr">
         <is>
           <t>TBD per service inventory</t>
         </is>
       </c>
-      <c r="I12" s="7" t="inlineStr">
+      <c r="I12" s="6" t="inlineStr">
         <is>
           <t>TBD</t>
         </is>
       </c>
-      <c r="J12" s="7" t="inlineStr">
+      <c r="J12" s="6" t="inlineStr">
         <is>
           <t>TBD</t>
         </is>
       </c>
-      <c r="K12" s="7" t="inlineStr">
+      <c r="K12" s="6" t="inlineStr">
         <is>
           <t>Verified manually executable</t>
         </is>
       </c>
-      <c r="L12" s="7" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="M12" s="7" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="N12" s="7" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="O12" s="7" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="P12" s="7" t="inlineStr">
+      <c r="L12" s="6" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="M12" s="6" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="N12" s="6" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="O12" s="6" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="P12" s="6" t="inlineStr">
         <is>
           <t>TBD</t>
         </is>
       </c>
-      <c r="Q12" s="7" t="inlineStr">
+      <c r="Q12" s="6" t="inlineStr">
         <is>
           <t>QC4 Stage1 Stage5</t>
         </is>
       </c>
-      <c r="R12" s="7" t="inlineStr">
+      <c r="R12" s="6" t="inlineStr">
         <is>
           <t>api-test-automation/universal/</t>
         </is>
       </c>
-      <c r="S12" s="7" t="inlineStr">
+      <c r="S12" s="6" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="T12" s="7" t="inlineStr">
+      <c r="T12" s="6" t="inlineStr">
         <is>
           <t>Verified manually executable</t>
         </is>
       </c>
-      <c r="U12" s="7" t="inlineStr">
+      <c r="U12" s="6" t="inlineStr">
         <is>
           <t>Not all modules on GitLab schedule</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="7" t="inlineStr">
+      <c r="A13" s="6" t="inlineStr">
         <is>
           <t>Universal Platform</t>
         </is>
       </c>
-      <c r="B13" s="7" t="inlineStr">
+      <c r="B13" s="6" t="inlineStr">
         <is>
           <t>UP API operations</t>
         </is>
       </c>
-      <c r="C13" s="7" t="inlineStr">
+      <c r="C13" s="6" t="inlineStr">
         <is>
           <t>API RestAssured</t>
         </is>
       </c>
-      <c r="D13" s="7" t="inlineStr">
+      <c r="D13" s="6" t="inlineStr">
         <is>
           <t>Enrollment IDP Withdrawal ops</t>
         </is>
       </c>
-      <c r="E13" s="7" t="inlineStr">
+      <c r="E13" s="6" t="inlineStr">
         <is>
           <t>api-test-automation</t>
         </is>
       </c>
-      <c r="F13" s="7" t="inlineStr">
+      <c r="F13" s="6" t="inlineStr">
         <is>
           <t>universal modules</t>
         </is>
       </c>
-      <c r="G13" s="7" t="inlineStr">
+      <c r="G13" s="6" t="inlineStr">
         <is>
           <t>11 unique HTTP operations per UP ledger</t>
         </is>
       </c>
-      <c r="H13" s="7" t="inlineStr">
+      <c r="H13" s="6" t="inlineStr">
         <is>
           <t>TBD full service catalog</t>
         </is>
       </c>
-      <c r="I13" s="7" t="inlineStr">
+      <c r="I13" s="6" t="inlineStr">
         <is>
           <t>11</t>
         </is>
       </c>
-      <c r="J13" s="7" t="inlineStr">
+      <c r="J13" s="6" t="inlineStr">
         <is>
           <t>TBD</t>
         </is>
       </c>
-      <c r="K13" s="7" t="inlineStr">
+      <c r="K13" s="6" t="inlineStr">
         <is>
           <t>Verified manually executable</t>
         </is>
       </c>
-      <c r="L13" s="7" t="inlineStr">
+      <c r="L13" s="6" t="inlineStr">
         <is>
           <t>Partial (metadataweb only scheduled)</t>
         </is>
       </c>
-      <c r="M13" s="7" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="N13" s="7" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="O13" s="7" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="P13" s="7" t="inlineStr">
+      <c r="M13" s="6" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="N13" s="6" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="O13" s="6" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="P13" s="6" t="inlineStr">
         <is>
           <t>TBD</t>
         </is>
       </c>
-      <c r="Q13" s="7" t="inlineStr">
+      <c r="Q13" s="6" t="inlineStr">
         <is>
           <t>Stage1</t>
         </is>
       </c>
-      <c r="R13" s="7" t="inlineStr">
+      <c r="R13" s="6" t="inlineStr">
         <is>
           <t>universal-platform-coverage/01-analysis/csv/api-operation-mapping.csv</t>
         </is>
       </c>
-      <c r="S13" s="7" t="inlineStr">
+      <c r="S13" s="6" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="T13" s="7" t="inlineStr">
+      <c r="T13" s="6" t="inlineStr">
         <is>
           <t>Verified manually executable</t>
         </is>
       </c>
-      <c r="U13" s="7" t="inlineStr">
+      <c r="U13" s="6" t="inlineStr">
         <is>
           <t>Denominator for full GS API surface not reconciled</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="7" t="inlineStr">
+      <c r="A14" s="6" t="inlineStr">
         <is>
           <t>ASTRO</t>
         </is>
       </c>
-      <c r="B14" s="7" t="inlineStr">
+      <c r="B14" s="6" t="inlineStr">
         <is>
           <t>ASTRO API</t>
         </is>
       </c>
-      <c r="C14" s="7" t="inlineStr">
+      <c r="C14" s="6" t="inlineStr">
         <is>
           <t>API TestNG</t>
         </is>
       </c>
-      <c r="D14" s="7" t="inlineStr">
+      <c r="D14" s="6" t="inlineStr">
         <is>
           <t>jsonapi-astro</t>
         </is>
       </c>
-      <c r="E14" s="7" t="inlineStr">
+      <c r="E14" s="6" t="inlineStr">
         <is>
           <t>api-test-automation</t>
         </is>
       </c>
-      <c r="F14" s="7" t="inlineStr">
+      <c r="F14" s="6" t="inlineStr">
         <is>
           <t>astro module</t>
         </is>
       </c>
-      <c r="G14" s="7" t="inlineStr">
+      <c r="G14" s="6" t="inlineStr">
         <is>
           <t>5 test classes</t>
         </is>
       </c>
-      <c r="H14" s="7" t="inlineStr">
+      <c r="H14" s="6" t="inlineStr">
         <is>
           <t>TBD</t>
         </is>
       </c>
-      <c r="I14" s="7" t="inlineStr">
+      <c r="I14" s="6" t="inlineStr">
         <is>
           <t>TBD</t>
         </is>
       </c>
-      <c r="J14" s="7" t="inlineStr">
+      <c r="J14" s="6" t="inlineStr">
         <is>
           <t>TBD</t>
         </is>
       </c>
-      <c r="K14" s="7" t="inlineStr">
+      <c r="K14" s="6" t="inlineStr">
         <is>
           <t>Verified manually executable</t>
         </is>
       </c>
-      <c r="L14" s="7" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="M14" s="7" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="N14" s="7" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="O14" s="7" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="P14" s="7" t="inlineStr">
+      <c r="L14" s="6" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="M14" s="6" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="N14" s="6" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="O14" s="6" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="P14" s="6" t="inlineStr">
         <is>
           <t>TBD</t>
         </is>
       </c>
-      <c r="Q14" s="7" t="inlineStr">
+      <c r="Q14" s="6" t="inlineStr">
         <is>
           <t>TBD</t>
         </is>
       </c>
-      <c r="R14" s="7" t="inlineStr">
+      <c r="R14" s="6" t="inlineStr">
         <is>
           <t>api-test-automation/astro/</t>
         </is>
       </c>
-      <c r="S14" s="7" t="inlineStr">
+      <c r="S14" s="6" t="inlineStr">
         <is>
           <t>Low</t>
         </is>
       </c>
-      <c r="T14" s="7" t="inlineStr">
+      <c r="T14" s="6" t="inlineStr">
         <is>
           <t>Verified manually executable</t>
         </is>
       </c>
-      <c r="U14" s="7" t="inlineStr">
+      <c r="U14" s="6" t="inlineStr">
         <is>
           <t>Scope vs GS priority TBD</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="7" t="inlineStr">
+      <c r="A15" s="6" t="inlineStr">
         <is>
           <t>Performance</t>
         </is>
       </c>
-      <c r="B15" s="7" t="inlineStr">
+      <c r="B15" s="6" t="inlineStr">
         <is>
           <t>Universal Platform</t>
         </is>
       </c>
-      <c r="C15" s="7" t="inlineStr">
+      <c r="C15" s="6" t="inlineStr">
         <is>
           <t>Performance JMeter Taurus</t>
         </is>
       </c>
-      <c r="D15" s="7" t="inlineStr">
+      <c r="D15" s="6" t="inlineStr">
         <is>
           <t>Enrollment IDP journeys</t>
         </is>
       </c>
-      <c r="E15" s="7" t="inlineStr">
+      <c r="E15" s="6" t="inlineStr">
         <is>
           <t>performance-test-automation</t>
         </is>
       </c>
-      <c r="F15" s="7" t="inlineStr">
+      <c r="F15" s="6" t="inlineStr">
         <is>
           <t>universal-platform/**/*.jmx</t>
         </is>
       </c>
-      <c r="G15" s="7" t="inlineStr">
+      <c r="G15" s="6" t="inlineStr">
         <is>
           <t>15 in-scope journeys per UP ledger</t>
         </is>
       </c>
-      <c r="H15" s="7" t="inlineStr">
+      <c r="H15" s="6" t="inlineStr">
         <is>
           <t>36 JMX / 53 Taurus total assets</t>
         </is>
       </c>
-      <c r="I15" s="7" t="inlineStr">
+      <c r="I15" s="6" t="inlineStr">
         <is>
           <t>15</t>
         </is>
       </c>
-      <c r="J15" s="7" t="inlineStr">
+      <c r="J15" s="6" t="inlineStr">
         <is>
           <t>TBD journey-level</t>
         </is>
       </c>
-      <c r="K15" s="7" t="inlineStr">
+      <c r="K15" s="6" t="inlineStr">
         <is>
           <t>Verified manually executable</t>
         </is>
       </c>
-      <c r="L15" s="7" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="M15" s="7" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="N15" s="7" t="inlineStr">
+      <c r="L15" s="6" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="M15" s="6" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="N15" s="6" t="inlineStr">
         <is>
           <t>AGSUP_IDP_REGRESSION_SUITE (scheduled weekdays)</t>
         </is>
       </c>
-      <c r="O15" s="7" t="inlineStr">
+      <c r="O15" s="6" t="inlineStr">
         <is>
           <t>Soft/informational perf</t>
         </is>
       </c>
-      <c r="P15" s="7" t="inlineStr">
+      <c r="P15" s="6" t="inlineStr">
         <is>
           <t>Both</t>
         </is>
       </c>
-      <c r="Q15" s="7" t="inlineStr">
+      <c r="Q15" s="6" t="inlineStr">
         <is>
           <t>QC4 Stage1</t>
         </is>
       </c>
-      <c r="R15" s="7" t="inlineStr">
+      <c r="R15" s="6" t="inlineStr">
         <is>
           <t>mobile2-api-db-validation/docs/01-shared/unite-msc-performance-testing-tracker.md</t>
         </is>
       </c>
-      <c r="S15" s="7" t="inlineStr">
+      <c r="S15" s="6" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="T15" s="7" t="inlineStr">
+      <c r="T15" s="6" t="inlineStr">
         <is>
           <t>Verified recurring regression (IDP perf only)</t>
         </is>
       </c>
-      <c r="U15" s="7" t="inlineStr">
+      <c r="U15" s="6" t="inlineStr">
         <is>
           <t>UP enrollment perf journeys not all scheduled</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="7" t="inlineStr">
+      <c r="A16" s="6" t="inlineStr">
         <is>
           <t>Performance</t>
         </is>
       </c>
-      <c r="B16" s="7" t="inlineStr">
+      <c r="B16" s="6" t="inlineStr">
         <is>
           <t>Unite MSC</t>
         </is>
       </c>
-      <c r="C16" s="7" t="inlineStr">
+      <c r="C16" s="6" t="inlineStr">
         <is>
           <t>Performance JMeter Taurus</t>
         </is>
       </c>
-      <c r="D16" s="7" t="inlineStr">
+      <c r="D16" s="6" t="inlineStr">
         <is>
           <t>MSC login core GET endpoints</t>
         </is>
       </c>
-      <c r="E16" s="7" t="inlineStr">
+      <c r="E16" s="6" t="inlineStr">
         <is>
           <t>performance-test-automation</t>
         </is>
       </c>
-      <c r="F16" s="7" t="inlineStr">
+      <c r="F16" s="6" t="inlineStr">
         <is>
           <t>mobile/unite-msc/jmeter</t>
         </is>
       </c>
-      <c r="G16" s="7" t="inlineStr">
+      <c r="G16" s="6" t="inlineStr">
         <is>
           <t>6 JMX + YAML pairs</t>
         </is>
       </c>
-      <c r="H16" s="7" t="inlineStr">
+      <c r="H16" s="6" t="inlineStr">
         <is>
           <t>TBD MSC journey catalog</t>
         </is>
       </c>
-      <c r="I16" s="7" t="inlineStr">
+      <c r="I16" s="6" t="inlineStr">
         <is>
           <t>3+ verified scripts</t>
         </is>
       </c>
-      <c r="J16" s="7" t="inlineStr">
+      <c r="J16" s="6" t="inlineStr">
         <is>
           <t>TBD</t>
         </is>
       </c>
-      <c r="K16" s="7" t="inlineStr">
+      <c r="K16" s="6" t="inlineStr">
         <is>
           <t>Verified manually executable</t>
         </is>
       </c>
-      <c r="L16" s="7" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="M16" s="7" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="N16" s="7" t="inlineStr">
+      <c r="L16" s="6" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="M16" s="6" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="N16" s="6" t="inlineStr">
         <is>
           <t>AGSUP_UNITE_MSC_ENDURANCE (manual)</t>
         </is>
       </c>
-      <c r="O16" s="7" t="inlineStr">
+      <c r="O16" s="6" t="inlineStr">
         <is>
           <t>Manual only</t>
         </is>
       </c>
-      <c r="P16" s="7" t="inlineStr">
+      <c r="P16" s="6" t="inlineStr">
         <is>
           <t>Non-IDP verified; IDP in progress</t>
         </is>
       </c>
-      <c r="Q16" s="7" t="inlineStr">
+      <c r="Q16" s="6" t="inlineStr">
         <is>
           <t>QC4 Stage1</t>
         </is>
       </c>
-      <c r="R16" s="7" t="inlineStr">
+      <c r="R16" s="6" t="inlineStr">
         <is>
           <t>performance/mobile/unite-msc/</t>
         </is>
       </c>
-      <c r="S16" s="7" t="inlineStr">
+      <c r="S16" s="6" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="T16" s="7" t="inlineStr">
+      <c r="T16" s="6" t="inlineStr">
         <is>
           <t>Verified manually executable — not scheduled</t>
         </is>
       </c>
-      <c r="U16" s="7" t="inlineStr">
+      <c r="U16" s="6" t="inlineStr">
         <is>
           <t>No periodic MSC perf trigger confirmed 2026-07-02</t>
         </is>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="7" t="inlineStr">
+      <c r="A17" s="6" t="inlineStr">
         <is>
           <t>Performance</t>
         </is>
       </c>
-      <c r="B17" s="7" t="inlineStr">
+      <c r="B17" s="6" t="inlineStr">
         <is>
           <t>Unite legacy</t>
         </is>
       </c>
-      <c r="C17" s="7" t="inlineStr">
+      <c r="C17" s="6" t="inlineStr">
         <is>
           <t>Performance JMeter</t>
         </is>
       </c>
-      <c r="D17" s="7" t="inlineStr">
+      <c r="D17" s="6" t="inlineStr">
         <is>
           <t>Legacy login</t>
         </is>
       </c>
-      <c r="E17" s="7" t="inlineStr">
+      <c r="E17" s="6" t="inlineStr">
         <is>
           <t>performance-test-automation</t>
         </is>
       </c>
-      <c r="F17" s="7" t="inlineStr">
+      <c r="F17" s="6" t="inlineStr">
         <is>
           <t>unite/legacy-login</t>
         </is>
       </c>
-      <c r="G17" s="7" t="inlineStr">
+      <c r="G17" s="6" t="inlineStr">
         <is>
           <t>1 JMX</t>
         </is>
       </c>
-      <c r="H17" s="7" t="inlineStr">
+      <c r="H17" s="6" t="inlineStr">
         <is>
           <t>TBD</t>
         </is>
       </c>
-      <c r="I17" s="7" t="inlineStr">
+      <c r="I17" s="6" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="J17" s="7" t="inlineStr">
+      <c r="J17" s="6" t="inlineStr">
         <is>
           <t>TBD</t>
         </is>
       </c>
-      <c r="K17" s="7" t="inlineStr">
+      <c r="K17" s="6" t="inlineStr">
         <is>
           <t>Verified manually executable</t>
         </is>
       </c>
-      <c r="L17" s="7" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="M17" s="7" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="N17" s="7" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="O17" s="7" t="inlineStr">
+      <c r="L17" s="6" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="M17" s="6" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="N17" s="6" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="O17" s="6" t="inlineStr">
         <is>
           <t>Manual</t>
         </is>
       </c>
-      <c r="P17" s="7" t="inlineStr">
+      <c r="P17" s="6" t="inlineStr">
         <is>
           <t>TBD</t>
         </is>
       </c>
-      <c r="Q17" s="7" t="inlineStr">
+      <c r="Q17" s="6" t="inlineStr">
         <is>
           <t>TBD</t>
         </is>
       </c>
-      <c r="R17" s="7" t="inlineStr">
+      <c r="R17" s="6" t="inlineStr">
         <is>
           <t>performance/unite/legacy-login/</t>
         </is>
       </c>
-      <c r="S17" s="7" t="inlineStr">
+      <c r="S17" s="6" t="inlineStr">
         <is>
           <t>Low</t>
         </is>
       </c>
-      <c r="T17" s="7" t="inlineStr">
+      <c r="T17" s="6" t="inlineStr">
         <is>
           <t>Verified manually executable</t>
         </is>
       </c>
-      <c r="U17" s="7" t="inlineStr">
+      <c r="U17" s="6" t="inlineStr">
         <is>
           <t>Adjacent to MSC</t>
         </is>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="7" t="inlineStr">
+      <c r="A18" s="6" t="inlineStr">
         <is>
           <t>Unite MSC</t>
         </is>
       </c>
-      <c r="B18" s="7" t="inlineStr">
+      <c r="B18" s="6" t="inlineStr">
         <is>
           <t>Microservice BDD</t>
         </is>
       </c>
-      <c r="C18" s="7" t="inlineStr">
+      <c r="C18" s="6" t="inlineStr">
         <is>
           <t>Service Cucumber JUnit</t>
         </is>
       </c>
-      <c r="D18" s="7" t="inlineStr">
+      <c r="D18" s="6" t="inlineStr">
         <is>
           <t>Per-microservice acceptance</t>
         </is>
       </c>
-      <c r="E18" s="7" t="inlineStr">
+      <c r="E18" s="6" t="inlineStr">
         <is>
           <t>UniteMSC 14 repos</t>
         </is>
       </c>
-      <c r="F18" s="7" t="inlineStr">
+      <c r="F18" s="6" t="inlineStr">
         <is>
           <t>features/*.feature</t>
         </is>
       </c>
-      <c r="G18" s="7" t="inlineStr">
+      <c r="G18" s="6" t="inlineStr">
         <is>
           <t>112+ Cucumber features aggregate</t>
         </is>
       </c>
-      <c r="H18" s="7" t="inlineStr">
+      <c r="H18" s="6" t="inlineStr">
         <is>
           <t>TBD BFF acceptance scope</t>
         </is>
       </c>
-      <c r="I18" s="7" t="inlineStr">
+      <c r="I18" s="6" t="inlineStr">
         <is>
           <t>N/A</t>
         </is>
       </c>
-      <c r="J18" s="7" t="inlineStr">
+      <c r="J18" s="6" t="inlineStr">
         <is>
           <t>N/A</t>
         </is>
       </c>
-      <c r="K18" s="7" t="inlineStr">
+      <c r="K18" s="6" t="inlineStr">
         <is>
           <t>Service CI via GitLab templates</t>
         </is>
       </c>
-      <c r="L18" s="7" t="inlineStr">
+      <c r="L18" s="6" t="inlineStr">
         <is>
           <t>Per-repo pipeline</t>
         </is>
       </c>
-      <c r="M18" s="7" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="N18" s="7" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="O18" s="7" t="inlineStr">
+      <c r="M18" s="6" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="N18" s="6" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="O18" s="6" t="inlineStr">
         <is>
           <t>Build/test gate on service deploy</t>
         </is>
       </c>
-      <c r="P18" s="7" t="inlineStr">
+      <c r="P18" s="6" t="inlineStr">
         <is>
           <t>Both</t>
         </is>
       </c>
-      <c r="Q18" s="7" t="inlineStr">
+      <c r="Q18" s="6" t="inlineStr">
         <is>
           <t>Dev/test</t>
         </is>
       </c>
-      <c r="R18" s="7" t="inlineStr">
+      <c r="R18" s="6" t="inlineStr">
         <is>
           <t>unite-mobile2/src/test/resources/features/</t>
         </is>
       </c>
-      <c r="S18" s="7" t="inlineStr">
+      <c r="S18" s="6" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="T18" s="7" t="inlineStr">
+      <c r="T18" s="6" t="inlineStr">
         <is>
           <t>Verified deployment validation</t>
         </is>
       </c>
-      <c r="U18" s="7" t="inlineStr">
+      <c r="U18" s="6" t="inlineStr">
         <is>
           <t>Not substitute for api-test-automation BFF tests</t>
         </is>
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="7" t="inlineStr">
+      <c r="A19" s="6" t="inlineStr">
         <is>
           <t>Mobile MSC</t>
         </is>
       </c>
-      <c r="B19" s="7" t="inlineStr">
+      <c r="B19" s="6" t="inlineStr">
         <is>
           <t>Account owner app</t>
         </is>
       </c>
-      <c r="C19" s="7" t="inlineStr">
+      <c r="C19" s="6" t="inlineStr">
         <is>
           <t>Angular Karma</t>
         </is>
       </c>
-      <c r="D19" s="7" t="inlineStr">
+      <c r="D19" s="6" t="inlineStr">
         <is>
           <t>Micro1 mobile app unit</t>
         </is>
       </c>
-      <c r="E19" s="7" t="inlineStr">
+      <c r="E19" s="6" t="inlineStr">
         <is>
           <t>unite-accountowner</t>
         </is>
       </c>
-      <c r="F19" s="7" t="inlineStr">
+      <c r="F19" s="6" t="inlineStr">
         <is>
           <t>*.spec.ts</t>
         </is>
       </c>
-      <c r="G19" s="7" t="inlineStr">
+      <c r="G19" s="6" t="inlineStr">
         <is>
           <t>120 spec files</t>
         </is>
       </c>
-      <c r="H19" s="7" t="inlineStr">
+      <c r="H19" s="6" t="inlineStr">
         <is>
           <t>TBD</t>
         </is>
       </c>
-      <c r="I19" s="7" t="inlineStr">
+      <c r="I19" s="6" t="inlineStr">
         <is>
           <t>TBD</t>
         </is>
       </c>
-      <c r="J19" s="7" t="inlineStr">
+      <c r="J19" s="6" t="inlineStr">
         <is>
           <t>120</t>
         </is>
       </c>
-      <c r="K19" s="7" t="inlineStr">
+      <c r="K19" s="6" t="inlineStr">
         <is>
           <t>TBD</t>
         </is>
       </c>
-      <c r="L19" s="7" t="inlineStr">
+      <c r="L19" s="6" t="inlineStr">
         <is>
           <t>CI on branch push</t>
         </is>
       </c>
-      <c r="M19" s="7" t="inlineStr">
+      <c r="M19" s="6" t="inlineStr">
         <is>
           <t>accountowner_build_tdd</t>
         </is>
       </c>
-      <c r="N19" s="7" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="O19" s="7" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="P19" s="7" t="inlineStr">
+      <c r="N19" s="6" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="O19" s="6" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="P19" s="6" t="inlineStr">
         <is>
           <t>Build gate not full GS regression</t>
         </is>
       </c>
-      <c r="Q19" s="7" t="inlineStr">
+      <c r="Q19" s="6" t="inlineStr">
         <is>
           <t>N/A</t>
         </is>
       </c>
-      <c r="R19" s="7" t="inlineStr">
+      <c r="R19" s="6" t="inlineStr">
         <is>
           <t>N/A</t>
         </is>
       </c>
-      <c r="S19" s="7" t="inlineStr">
+      <c r="S19" s="6" t="inlineStr">
         <is>
           <t>UniteMSC/unite-accountowner/</t>
         </is>
       </c>
-      <c r="T19" s="7" t="inlineStr">
+      <c r="T19" s="6" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="U19" s="7" t="inlineStr">
+      <c r="U19" s="6" t="inlineStr">
         <is>
           <t>Verified deployment validation</t>
         </is>
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="7" t="inlineStr">
+      <c r="A20" s="6" t="inlineStr">
         <is>
           <t>COPACS</t>
         </is>
       </c>
-      <c r="B20" s="7" t="inlineStr">
+      <c r="B20" s="6" t="inlineStr">
         <is>
           <t>Platform</t>
         </is>
       </c>
-      <c r="C20" s="7" t="inlineStr">
+      <c r="C20" s="6" t="inlineStr">
         <is>
           <t>TBD</t>
         </is>
       </c>
-      <c r="D20" s="7" t="inlineStr">
+      <c r="D20" s="6" t="inlineStr">
         <is>
           <t>TBD</t>
         </is>
       </c>
-      <c r="E20" s="7" t="inlineStr">
+      <c r="E20" s="6" t="inlineStr">
         <is>
           <t>Not identified in reviewed repos</t>
         </is>
       </c>
-      <c r="F20" s="7" t="inlineStr">
+      <c r="F20" s="6" t="inlineStr">
         <is>
           <t>TBD</t>
         </is>
       </c>
-      <c r="G20" s="7" t="inlineStr">
+      <c r="G20" s="6" t="inlineStr">
         <is>
           <t>TBD</t>
         </is>
       </c>
-      <c r="H20" s="7" t="inlineStr">
+      <c r="H20" s="6" t="inlineStr">
         <is>
           <t>TBD</t>
         </is>
       </c>
-      <c r="I20" s="7" t="inlineStr">
+      <c r="I20" s="6" t="inlineStr">
         <is>
           <t>TBD</t>
         </is>
       </c>
-      <c r="J20" s="7" t="inlineStr">
+      <c r="J20" s="6" t="inlineStr">
         <is>
           <t>TBD</t>
         </is>
       </c>
-      <c r="K20" s="7" t="inlineStr">
+      <c r="K20" s="6" t="inlineStr">
         <is>
           <t>No validated automation identified</t>
         </is>
       </c>
-      <c r="L20" s="7" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="M20" s="7" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="N20" s="7" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="O20" s="7" t="inlineStr">
+      <c r="L20" s="6" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="M20" s="6" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="N20" s="6" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="O20" s="6" t="inlineStr">
         <is>
           <t>None</t>
         </is>
       </c>
-      <c r="P20" s="7" t="inlineStr">
+      <c r="P20" s="6" t="inlineStr">
         <is>
           <t>TBD</t>
         </is>
       </c>
-      <c r="Q20" s="7" t="inlineStr">
+      <c r="Q20" s="6" t="inlineStr">
         <is>
           <t>TBD</t>
         </is>
       </c>
-      <c r="R20" s="7" t="inlineStr">
+      <c r="R20" s="6" t="inlineStr">
         <is>
           <t>N/A</t>
         </is>
       </c>
-      <c r="S20" s="7" t="inlineStr">
+      <c r="S20" s="6" t="inlineStr">
         <is>
           <t>Low</t>
         </is>
       </c>
-      <c r="T20" s="7" t="inlineStr">
+      <c r="T20" s="6" t="inlineStr">
         <is>
           <t>No validated automation identified</t>
         </is>
       </c>
-      <c r="U20" s="7" t="inlineStr">
+      <c r="U20" s="6" t="inlineStr">
         <is>
           <t>Requires scope confirmation from business owners</t>
         </is>
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="7" t="inlineStr">
+      <c r="A21" s="6" t="inlineStr">
         <is>
           <t>Government Savings</t>
         </is>
       </c>
-      <c r="B21" s="7" t="inlineStr">
+      <c r="B21" s="6" t="inlineStr">
         <is>
           <t>Application code coverage</t>
         </is>
       </c>
-      <c r="C21" s="7" t="inlineStr">
+      <c r="C21" s="6" t="inlineStr">
         <is>
           <t>JaCoCo Sonar</t>
         </is>
       </c>
-      <c r="D21" s="7" t="inlineStr">
+      <c r="D21" s="6" t="inlineStr">
         <is>
           <t>Service unit coverage</t>
         </is>
       </c>
-      <c r="E21" s="7" t="inlineStr">
+      <c r="E21" s="6" t="inlineStr">
         <is>
           <t>UniteMSC microservice repos</t>
         </is>
       </c>
-      <c r="F21" s="7" t="inlineStr">
+      <c r="F21" s="6" t="inlineStr">
         <is>
           <t>POM jacoco config</t>
         </is>
       </c>
-      <c r="G21" s="7" t="inlineStr">
+      <c r="G21" s="6" t="inlineStr">
         <is>
           <t>Service unit tests</t>
         </is>
       </c>
-      <c r="H21" s="7" t="inlineStr">
+      <c r="H21" s="6" t="inlineStr">
         <is>
           <t>TBD</t>
         </is>
       </c>
-      <c r="I21" s="7" t="inlineStr">
+      <c r="I21" s="6" t="inlineStr">
         <is>
           <t>TBD</t>
         </is>
       </c>
-      <c r="J21" s="7" t="inlineStr">
+      <c r="J21" s="6" t="inlineStr">
         <is>
           <t>N/A</t>
         </is>
       </c>
-      <c r="K21" s="7" t="inlineStr">
+      <c r="K21" s="6" t="inlineStr">
         <is>
           <t>N/A</t>
         </is>
       </c>
-      <c r="L21" s="7" t="inlineStr">
+      <c r="L21" s="6" t="inlineStr">
         <is>
           <t>Service pipeline</t>
         </is>
       </c>
-      <c r="M21" s="7" t="inlineStr">
+      <c r="M21" s="6" t="inlineStr">
         <is>
           <t>GitLab shared templates</t>
         </is>
       </c>
-      <c r="N21" s="7" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="O21" s="7" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="P21" s="7" t="inlineStr">
+      <c r="N21" s="6" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="O21" s="6" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="P21" s="6" t="inlineStr">
         <is>
           <t>Sonar disabled RUN_SONARQUBE false</t>
         </is>
       </c>
-      <c r="Q21" s="7" t="inlineStr">
+      <c r="Q21" s="6" t="inlineStr">
         <is>
           <t>NA</t>
         </is>
       </c>
-      <c r="R21" s="7" t="inlineStr">
+      <c r="R21" s="6" t="inlineStr">
         <is>
           <t>NA</t>
         </is>
       </c>
-      <c r="S21" s="7" t="inlineStr">
+      <c r="S21" s="6" t="inlineStr">
         <is>
           <t>unite-mobile1/pom.xml</t>
         </is>
       </c>
-      <c r="T21" s="7" t="inlineStr">
+      <c r="T21" s="6" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="U21" s="7" t="inlineStr">
+      <c r="U21" s="6" t="inlineStr">
         <is>
           <t>Not a QA regression gate</t>
         </is>
@@ -3230,1140 +3338,1140 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="7" t="inlineStr">
+      <c r="A2" s="6" t="inlineStr">
         <is>
           <t>GitLab</t>
         </is>
       </c>
-      <c r="B2" s="7" t="inlineStr">
+      <c r="B2" s="6" t="inlineStr">
         <is>
           <t>prepare</t>
         </is>
       </c>
-      <c r="C2" s="7" t="inlineStr">
+      <c r="C2" s="6" t="inlineStr">
         <is>
           <t>api-test-automation</t>
         </is>
       </c>
-      <c r="D2" s="7" t="inlineStr">
+      <c r="D2" s="6" t="inlineStr">
         <is>
           <t>Pipeline default</t>
         </is>
       </c>
-      <c r="E2" s="7" t="inlineStr">
+      <c r="E2" s="6" t="inlineStr">
         <is>
           <t>On push/MR</t>
         </is>
       </c>
-      <c r="F2" s="7" t="inlineStr">
+      <c r="F2" s="6" t="inlineStr">
         <is>
           <t>Stage1 DB props</t>
         </is>
       </c>
-      <c r="G2" s="7" t="inlineStr">
+      <c r="G2" s="6" t="inlineStr">
         <is>
           <t>Secure files setup</t>
         </is>
       </c>
-      <c r="H2" s="7" t="inlineStr">
+      <c r="H2" s="6" t="inlineStr">
         <is>
           <t>N/A</t>
         </is>
       </c>
-      <c r="I2" s="7" t="inlineStr">
+      <c r="I2" s="6" t="inlineStr">
         <is>
           <t>env_variables.env dotenv</t>
         </is>
       </c>
-      <c r="J2" s="7" t="inlineStr">
+      <c r="J2" s="6" t="inlineStr">
         <is>
           <t>Non-blocking prep</t>
         </is>
       </c>
-      <c r="K2" s="7" t="inlineStr">
+      <c r="K2" s="6" t="inlineStr">
         <is>
           <t>Informational</t>
         </is>
       </c>
-      <c r="L2" s="7" t="inlineStr">
+      <c r="L2" s="6" t="inlineStr">
         <is>
           <t>api-test-automation/.gitlab-ci.yml</t>
         </is>
       </c>
-      <c r="M2" s="7" t="inlineStr">
+      <c r="M2" s="6" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="N2" s="7" t="inlineStr">
+      <c r="N2" s="6" t="inlineStr">
         <is>
           <t>All scheduled jobs depend on secure files</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="7" t="inlineStr">
+      <c r="A3" s="6" t="inlineStr">
         <is>
           <t>GitLab</t>
         </is>
       </c>
-      <c r="B3" s="7" t="inlineStr">
+      <c r="B3" s="6" t="inlineStr">
         <is>
           <t>scheduled_metadataweb_stage1</t>
         </is>
       </c>
-      <c r="C3" s="7" t="inlineStr">
+      <c r="C3" s="6" t="inlineStr">
         <is>
           <t>api-test-automation</t>
         </is>
       </c>
-      <c r="D3" s="7" t="inlineStr">
+      <c r="D3" s="6" t="inlineStr">
         <is>
           <t>only: schedules</t>
         </is>
       </c>
-      <c r="E3" s="7" t="inlineStr">
+      <c r="E3" s="6" t="inlineStr">
         <is>
           <t>Nightly (~1 AM per comment — schedule ID not verified in this pass)</t>
         </is>
       </c>
-      <c r="F3" s="7" t="inlineStr">
+      <c r="F3" s="6" t="inlineStr">
         <is>
           <t>Stage1</t>
         </is>
       </c>
-      <c r="G3" s="7" t="inlineStr">
+      <c r="G3" s="6" t="inlineStr">
         <is>
           <t>stage1-api-metadata-pipeline</t>
         </is>
       </c>
-      <c r="H3" s="7" t="inlineStr">
+      <c r="H3" s="6" t="inlineStr">
         <is>
           <t>Universal metadataweb API</t>
         </is>
       </c>
-      <c r="I3" s="7" t="inlineStr">
+      <c r="I3" s="6" t="inlineStr">
         <is>
           <t>JUnit surefire</t>
         </is>
       </c>
-      <c r="J3" s="7" t="inlineStr">
+      <c r="J3" s="6" t="inlineStr">
         <is>
           <t>exit non-zero on test fail</t>
         </is>
       </c>
-      <c r="K3" s="7" t="inlineStr">
+      <c r="K3" s="6" t="inlineStr">
         <is>
           <t>Hard gate (scheduled job)</t>
         </is>
       </c>
-      <c r="L3" s="7" t="inlineStr">
+      <c r="L3" s="6" t="inlineStr">
         <is>
           <t>api-test-automation/.gitlab-ci.yml</t>
         </is>
       </c>
-      <c r="M3" s="7" t="inlineStr">
+      <c r="M3" s="6" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="N3" s="7" t="inlineStr">
+      <c r="N3" s="6" t="inlineStr">
         <is>
           <t>Only confirmed GS-related nightly in api-test-automation</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="7" t="inlineStr">
+      <c r="A4" s="6" t="inlineStr">
         <is>
           <t>GitLab</t>
         </is>
       </c>
-      <c r="B4" s="7" t="inlineStr">
+      <c r="B4" s="6" t="inlineStr">
         <is>
           <t>download_secure_files (include)</t>
         </is>
       </c>
-      <c r="C4" s="7" t="inlineStr">
+      <c r="C4" s="6" t="inlineStr">
         <is>
           <t>api-test-automation</t>
         </is>
       </c>
-      <c r="D4" s="7" t="inlineStr">
+      <c r="D4" s="6" t="inlineStr">
         <is>
           <t>From shared include</t>
         </is>
       </c>
-      <c r="E4" s="7" t="inlineStr">
+      <c r="E4" s="6" t="inlineStr">
         <is>
           <t>With prepare</t>
         </is>
       </c>
-      <c r="F4" s="7" t="inlineStr">
+      <c r="F4" s="6" t="inlineStr">
         <is>
           <t>N/A</t>
         </is>
       </c>
-      <c r="G4" s="7" t="inlineStr">
+      <c r="G4" s="6" t="inlineStr">
         <is>
           <t>N/A</t>
         </is>
       </c>
-      <c r="H4" s="7" t="inlineStr">
+      <c r="H4" s="6" t="inlineStr">
         <is>
           <t>N/A</t>
         </is>
       </c>
-      <c r="I4" s="7" t="inlineStr">
+      <c r="I4" s="6" t="inlineStr">
         <is>
           <t>secure files</t>
         </is>
       </c>
-      <c r="J4" s="7" t="inlineStr">
+      <c r="J4" s="6" t="inlineStr">
         <is>
           <t>Unknown</t>
         </is>
       </c>
-      <c r="K4" s="7" t="inlineStr">
+      <c r="K4" s="6" t="inlineStr">
         <is>
           <t>Dependency</t>
         </is>
       </c>
-      <c r="L4" s="7" t="inlineStr">
+      <c r="L4" s="6" t="inlineStr">
         <is>
           <t>include ascensus-gs/.../includes</t>
         </is>
       </c>
-      <c r="M4" s="7" t="inlineStr">
+      <c r="M4" s="6" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="N4" s="7" t="inlineStr">
+      <c r="N4" s="6" t="inlineStr">
         <is>
           <t>Job defined in external include project</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="7" t="inlineStr">
+      <c r="A5" s="6" t="inlineStr">
         <is>
           <t>GitLab</t>
         </is>
       </c>
-      <c r="B5" s="7" t="inlineStr">
+      <c r="B5" s="6" t="inlineStr">
         <is>
           <t>prepare</t>
         </is>
       </c>
-      <c r="C5" s="7" t="inlineStr">
+      <c r="C5" s="6" t="inlineStr">
         <is>
           <t>prime-test-automation</t>
         </is>
       </c>
-      <c r="D5" s="7" t="inlineStr">
+      <c r="D5" s="6" t="inlineStr">
         <is>
           <t>Pipeline default</t>
         </is>
       </c>
-      <c r="E5" s="7" t="inlineStr">
+      <c r="E5" s="6" t="inlineStr">
         <is>
           <t>On push/MR</t>
         </is>
       </c>
-      <c r="F5" s="7" t="inlineStr">
+      <c r="F5" s="6" t="inlineStr">
         <is>
           <t>Stage1</t>
         </is>
       </c>
-      <c r="G5" s="7" t="inlineStr">
+      <c r="G5" s="6" t="inlineStr">
         <is>
           <t>Secure files</t>
         </is>
       </c>
-      <c r="H5" s="7" t="inlineStr">
+      <c r="H5" s="6" t="inlineStr">
         <is>
           <t>N/A</t>
         </is>
       </c>
-      <c r="I5" s="7" t="inlineStr">
+      <c r="I5" s="6" t="inlineStr">
         <is>
           <t>artifacts</t>
         </is>
       </c>
-      <c r="J5" s="7" t="inlineStr">
+      <c r="J5" s="6" t="inlineStr">
         <is>
           <t>Prep</t>
         </is>
       </c>
-      <c r="K5" s="7" t="inlineStr">
+      <c r="K5" s="6" t="inlineStr">
         <is>
           <t>Informational</t>
         </is>
       </c>
-      <c r="L5" s="7" t="inlineStr">
+      <c r="L5" s="6" t="inlineStr">
         <is>
           <t>prime-test-automation/.gitlab-ci.yml</t>
         </is>
       </c>
-      <c r="M5" s="7" t="inlineStr">
+      <c r="M5" s="6" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="N5" s="7" t="inlineStr"/>
+      <c r="N5" s="6" t="inlineStr"/>
     </row>
     <row r="6">
-      <c r="A6" s="7" t="inlineStr">
+      <c r="A6" s="6" t="inlineStr">
         <is>
           <t>GitLab</t>
         </is>
       </c>
-      <c r="B6" s="7" t="inlineStr">
+      <c r="B6" s="6" t="inlineStr">
         <is>
           <t>scheduled_regression_job</t>
         </is>
       </c>
-      <c r="C6" s="7" t="inlineStr">
+      <c r="C6" s="6" t="inlineStr">
         <is>
           <t>prime-test-automation</t>
         </is>
       </c>
-      <c r="D6" s="7" t="inlineStr">
+      <c r="D6" s="6" t="inlineStr">
         <is>
           <t>only: schedules</t>
         </is>
       </c>
-      <c r="E6" s="7" t="inlineStr">
+      <c r="E6" s="6" t="inlineStr">
         <is>
           <t>Nightly (KB cites schedule #3961313 — not re-verified live)</t>
         </is>
       </c>
-      <c r="F6" s="7" t="inlineStr">
+      <c r="F6" s="6" t="inlineStr">
         <is>
           <t>Stage1</t>
         </is>
       </c>
-      <c r="G6" s="7" t="inlineStr">
+      <c r="G6" s="6" t="inlineStr">
         <is>
           <t>stage1-ue-regression-test + stage1-unite-regression-master</t>
         </is>
       </c>
-      <c r="H6" s="7" t="inlineStr">
+      <c r="H6" s="6" t="inlineStr">
         <is>
           <t>V3 UE + Unite core UI (IDP login contributions withdrawals CSR)</t>
         </is>
       </c>
-      <c r="I6" s="7" t="inlineStr">
+      <c r="I6" s="6" t="inlineStr">
         <is>
           <t>JUnit both modules</t>
         </is>
       </c>
-      <c r="J6" s="7" t="inlineStr">
+      <c r="J6" s="6" t="inlineStr">
         <is>
           <t>exit 1 if either phase fails</t>
         </is>
       </c>
-      <c r="K6" s="7" t="inlineStr">
+      <c r="K6" s="6" t="inlineStr">
         <is>
           <t>Hard gate (scheduled)</t>
         </is>
       </c>
-      <c r="L6" s="7" t="inlineStr">
+      <c r="L6" s="6" t="inlineStr">
         <is>
           <t>prime-test-automation/.gitlab-ci.yml</t>
         </is>
       </c>
-      <c r="M6" s="7" t="inlineStr">
+      <c r="M6" s="6" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="N6" s="7" t="inlineStr">
+      <c r="N6" s="6" t="inlineStr">
         <is>
           <t>Selenium chrome service; primary V3 GS UI nightly</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="7" t="inlineStr">
+      <c r="A7" s="6" t="inlineStr">
         <is>
           <t>GitLab</t>
         </is>
       </c>
-      <c r="B7" s="7" t="inlineStr">
+      <c r="B7" s="6" t="inlineStr">
         <is>
           <t>stage5_smoke_job</t>
         </is>
       </c>
-      <c r="C7" s="7" t="inlineStr">
+      <c r="C7" s="6" t="inlineStr">
         <is>
           <t>prime-test-automation</t>
         </is>
       </c>
-      <c r="D7" s="7" t="inlineStr">
+      <c r="D7" s="6" t="inlineStr">
         <is>
           <t>schedule when: manual</t>
         </is>
       </c>
-      <c r="E7" s="7" t="inlineStr">
+      <c r="E7" s="6" t="inlineStr">
         <is>
           <t>Manual</t>
         </is>
       </c>
-      <c r="F7" s="7" t="inlineStr">
+      <c r="F7" s="6" t="inlineStr">
         <is>
           <t>Stage5</t>
         </is>
       </c>
-      <c r="G7" s="7" t="inlineStr">
+      <c r="G7" s="6" t="inlineStr">
         <is>
           <t>stage5-smoke profiles</t>
         </is>
       </c>
-      <c r="H7" s="7" t="inlineStr">
+      <c r="H7" s="6" t="inlineStr">
         <is>
           <t>V3 lightweight smoke</t>
         </is>
       </c>
-      <c r="I7" s="7" t="inlineStr">
+      <c r="I7" s="6" t="inlineStr">
         <is>
           <t>JUnit</t>
         </is>
       </c>
-      <c r="J7" s="7" t="inlineStr">
+      <c r="J7" s="6" t="inlineStr">
         <is>
           <t>Unknown</t>
         </is>
       </c>
-      <c r="K7" s="7" t="inlineStr">
+      <c r="K7" s="6" t="inlineStr">
         <is>
           <t>Manual smoke</t>
         </is>
       </c>
-      <c r="L7" s="7" t="inlineStr">
+      <c r="L7" s="6" t="inlineStr">
         <is>
           <t>prime-test-automation/.gitlab-ci.yml</t>
         </is>
       </c>
-      <c r="M7" s="7" t="inlineStr">
+      <c r="M7" s="6" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="N7" s="7" t="inlineStr">
+      <c r="N7" s="6" t="inlineStr">
         <is>
           <t>Not recurring regression</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="7" t="inlineStr">
+      <c r="A8" s="6" t="inlineStr">
         <is>
           <t>GitLab</t>
         </is>
       </c>
-      <c r="B8" s="7" t="inlineStr">
+      <c r="B8" s="6" t="inlineStr">
         <is>
           <t>Per-microservice pipeline</t>
         </is>
       </c>
-      <c r="C8" s="7" t="inlineStr">
+      <c r="C8" s="6" t="inlineStr">
         <is>
           <t>UniteMSC (14 repos)</t>
         </is>
       </c>
-      <c r="D8" s="7" t="inlineStr">
+      <c r="D8" s="6" t="inlineStr">
         <is>
           <t>Push/MR</t>
         </is>
       </c>
-      <c r="E8" s="7" t="inlineStr">
+      <c r="E8" s="6" t="inlineStr">
         <is>
           <t>Per commit</t>
         </is>
       </c>
-      <c r="F8" s="7" t="inlineStr">
+      <c r="F8" s="6" t="inlineStr">
         <is>
           <t>Dev/test</t>
         </is>
       </c>
-      <c r="G8" s="7" t="inlineStr">
+      <c r="G8" s="6" t="inlineStr">
         <is>
           <t>Maven test + Cucumber</t>
         </is>
       </c>
-      <c r="H8" s="7" t="inlineStr">
+      <c r="H8" s="6" t="inlineStr">
         <is>
           <t>Service under test</t>
         </is>
       </c>
-      <c r="I8" s="7" t="inlineStr">
+      <c r="I8" s="6" t="inlineStr">
         <is>
           <t>Jacoco Cluecumber</t>
         </is>
       </c>
-      <c r="J8" s="7" t="inlineStr">
+      <c r="J8" s="6" t="inlineStr">
         <is>
           <t>Typical Maven fail blocks stage</t>
         </is>
       </c>
-      <c r="K8" s="7" t="inlineStr">
+      <c r="K8" s="6" t="inlineStr">
         <is>
           <t>Deployment/build gate</t>
         </is>
       </c>
-      <c r="L8" s="7" t="inlineStr">
+      <c r="L8" s="6" t="inlineStr">
         <is>
           <t>unite-mobile1/.gitlab-ci.yml + shared unitemsc_template.yml</t>
         </is>
       </c>
-      <c r="M8" s="7" t="inlineStr">
+      <c r="M8" s="6" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="N8" s="7" t="inlineStr">
+      <c r="N8" s="6" t="inlineStr">
         <is>
           <t>Exact job names in external template not in local clone</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="7" t="inlineStr">
+      <c r="A9" s="6" t="inlineStr">
         <is>
           <t>GitLab</t>
         </is>
       </c>
-      <c r="B9" s="7" t="inlineStr">
+      <c r="B9" s="6" t="inlineStr">
         <is>
           <t>accountowner_build_tdd</t>
         </is>
       </c>
-      <c r="C9" s="7" t="inlineStr">
+      <c r="C9" s="6" t="inlineStr">
         <is>
           <t>unite-accountowner</t>
         </is>
       </c>
-      <c r="D9" s="7" t="inlineStr">
+      <c r="D9" s="6" t="inlineStr">
         <is>
           <t>Branch push</t>
         </is>
       </c>
-      <c r="E9" s="7" t="inlineStr">
+      <c r="E9" s="6" t="inlineStr">
         <is>
           <t>Per commit</t>
         </is>
       </c>
-      <c r="F9" s="7" t="inlineStr">
+      <c r="F9" s="6" t="inlineStr">
         <is>
           <t>N/A</t>
         </is>
       </c>
-      <c r="G9" s="7" t="inlineStr">
+      <c r="G9" s="6" t="inlineStr">
         <is>
           <t>Angular build</t>
         </is>
       </c>
-      <c r="H9" s="7" t="inlineStr">
+      <c r="H9" s="6" t="inlineStr">
         <is>
           <t>Mobile account owner app</t>
         </is>
       </c>
-      <c r="I9" s="7" t="inlineStr">
+      <c r="I9" s="6" t="inlineStr">
         <is>
           <t>Build logs</t>
         </is>
       </c>
-      <c r="J9" s="7" t="inlineStr">
+      <c r="J9" s="6" t="inlineStr">
         <is>
           <t>Build fail blocks</t>
         </is>
       </c>
-      <c r="K9" s="7" t="inlineStr">
+      <c r="K9" s="6" t="inlineStr">
         <is>
           <t>Build gate</t>
         </is>
       </c>
-      <c r="L9" s="7" t="inlineStr">
+      <c r="L9" s="6" t="inlineStr">
         <is>
           <t>unite-accountowner/devops/templates/accountowner_tdd.yaml</t>
         </is>
       </c>
-      <c r="M9" s="7" t="inlineStr">
+      <c r="M9" s="6" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="N9" s="7" t="inlineStr">
+      <c r="N9" s="6" t="inlineStr">
         <is>
           <t>Not GS regression suite</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="7" t="inlineStr">
+      <c r="A10" s="6" t="inlineStr">
         <is>
           <t>GitHub Actions</t>
         </is>
       </c>
-      <c r="B10" s="7" t="inlineStr">
+      <c r="B10" s="6" t="inlineStr">
         <is>
           <t>Mobile2 Dashboard vertical slice</t>
         </is>
       </c>
-      <c r="C10" s="7" t="inlineStr">
+      <c r="C10" s="6" t="inlineStr">
         <is>
           <t>External deployment pipeline repo (not in audit clone)</t>
         </is>
       </c>
-      <c r="D10" s="7" t="inlineStr">
+      <c r="D10" s="6" t="inlineStr">
         <is>
           <t>Validated with Chaitanya</t>
         </is>
       </c>
-      <c r="E10" s="7" t="inlineStr">
+      <c r="E10" s="6" t="inlineStr">
         <is>
           <t>N/A</t>
         </is>
       </c>
-      <c r="F10" s="7" t="inlineStr">
+      <c r="F10" s="6" t="inlineStr">
         <is>
           <t>Nexus consume + dashboard profile</t>
         </is>
       </c>
-      <c r="G10" s="7" t="inlineStr">
+      <c r="G10" s="6" t="inlineStr">
         <is>
           <t>mobile-ms-dashboard-integration</t>
         </is>
       </c>
-      <c r="H10" s="7" t="inlineStr">
+      <c r="H10" s="6" t="inlineStr">
         <is>
           <t>Mobile 2 deployment validation</t>
         </is>
       </c>
-      <c r="I10" s="7" t="inlineStr">
+      <c r="I10" s="6" t="inlineStr">
         <is>
           <t>Nexus artifact + HTML report</t>
         </is>
       </c>
-      <c r="J10" s="7" t="inlineStr">
+      <c r="J10" s="6" t="inlineStr">
         <is>
           <t>N/A</t>
         </is>
       </c>
-      <c r="K10" s="7" t="inlineStr">
+      <c r="K10" s="6" t="inlineStr">
         <is>
           <t>N/A</t>
         </is>
       </c>
-      <c r="L10" s="7" t="inlineStr">
+      <c r="L10" s="6" t="inlineStr">
         <is>
           <t>Failure blocks workflow run (external)</t>
         </is>
       </c>
-      <c r="M10" s="7" t="inlineStr">
+      <c r="M10" s="6" t="inlineStr">
         <is>
           <t>Deployment validation — not GitLab nightly</t>
         </is>
       </c>
-      <c r="N10" s="7" t="inlineStr">
+      <c r="N10" s="6" t="inlineStr">
         <is>
           <t>Externally validated 2026-07</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="7" t="inlineStr">
+      <c r="A11" s="6" t="inlineStr">
         <is>
           <t>Jenkins</t>
         </is>
       </c>
-      <c r="B11" s="7" t="inlineStr">
+      <c r="B11" s="6" t="inlineStr">
         <is>
           <t>UNITE-TB-REFRESH</t>
         </is>
       </c>
-      <c r="C11" s="7" t="inlineStr">
+      <c r="C11" s="6" t="inlineStr">
         <is>
           <t>unite-test-automation</t>
         </is>
       </c>
-      <c r="D11" s="7" t="inlineStr">
+      <c r="D11" s="6" t="inlineStr">
         <is>
           <t>Ant build.xml reference</t>
         </is>
       </c>
-      <c r="E11" s="7" t="inlineStr">
+      <c r="E11" s="6" t="inlineStr">
         <is>
           <t>On demand / pre-regression</t>
         </is>
       </c>
-      <c r="F11" s="7" t="inlineStr">
+      <c r="F11" s="6" t="inlineStr">
         <is>
           <t>TB refresh</t>
         </is>
       </c>
-      <c r="G11" s="7" t="inlineStr">
+      <c r="G11" s="6" t="inlineStr">
         <is>
           <t>Testbed setup</t>
         </is>
       </c>
-      <c r="H11" s="7" t="inlineStr">
+      <c r="H11" s="6" t="inlineStr">
         <is>
           <t>V2 Unite</t>
         </is>
       </c>
-      <c r="I11" s="7" t="inlineStr">
+      <c r="I11" s="6" t="inlineStr">
         <is>
           <t>Logs</t>
         </is>
       </c>
-      <c r="J11" s="7" t="inlineStr">
+      <c r="J11" s="6" t="inlineStr">
         <is>
           <t>Unknown</t>
         </is>
       </c>
-      <c r="K11" s="7" t="inlineStr">
+      <c r="K11" s="6" t="inlineStr">
         <is>
           <t>Environment prep</t>
         </is>
       </c>
-      <c r="L11" s="7" t="inlineStr">
+      <c r="L11" s="6" t="inlineStr">
         <is>
           <t>unite/bin/build.xml</t>
         </is>
       </c>
-      <c r="M11" s="7" t="inlineStr">
+      <c r="M11" s="6" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="N11" s="7" t="inlineStr">
+      <c r="N11" s="6" t="inlineStr">
         <is>
           <t>devjenkinsnt1:8080</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="7" t="inlineStr">
+      <c r="A12" s="6" t="inlineStr">
         <is>
           <t>Jenkins</t>
         </is>
       </c>
-      <c r="B12" s="7" t="inlineStr">
+      <c r="B12" s="6" t="inlineStr">
         <is>
           <t>V2 regression Ant targets</t>
         </is>
       </c>
-      <c r="C12" s="7" t="inlineStr">
+      <c r="C12" s="6" t="inlineStr">
         <is>
           <t>unite-test-automation</t>
         </is>
       </c>
-      <c r="D12" s="7" t="inlineStr">
+      <c r="D12" s="6" t="inlineStr">
         <is>
           <t>Ant CLI / Jenkins job (name not in repo)</t>
         </is>
       </c>
-      <c r="E12" s="7" t="inlineStr">
+      <c r="E12" s="6" t="inlineStr">
         <is>
           <t>Daily/weekly targets documented</t>
         </is>
       </c>
-      <c r="F12" s="7" t="inlineStr">
+      <c r="F12" s="6" t="inlineStr">
         <is>
           <t>Stage1 Stage5</t>
         </is>
       </c>
-      <c r="G12" s="7" t="inlineStr">
+      <c r="G12" s="6" t="inlineStr">
         <is>
           <t>regression-frontoffice-daily regression-backoffice-daily stage1-*-regression</t>
         </is>
       </c>
-      <c r="H12" s="7" t="inlineStr">
+      <c r="H12" s="6" t="inlineStr">
         <is>
           <t>V2 Unite UI + backoffice</t>
         </is>
       </c>
-      <c r="I12" s="7" t="inlineStr">
+      <c r="I12" s="6" t="inlineStr">
         <is>
           <t>TestNG reports</t>
         </is>
       </c>
-      <c r="J12" s="7" t="inlineStr">
+      <c r="J12" s="6" t="inlineStr">
         <is>
           <t>Unknown</t>
         </is>
       </c>
-      <c r="K12" s="7" t="inlineStr">
+      <c r="K12" s="6" t="inlineStr">
         <is>
           <t>Soft/manual — job name TBD</t>
         </is>
       </c>
-      <c r="L12" s="7" t="inlineStr">
+      <c r="L12" s="6" t="inlineStr">
         <is>
           <t>unite/bin/build.xml</t>
         </is>
       </c>
-      <c r="M12" s="7" t="inlineStr">
+      <c r="M12" s="6" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="N12" s="7" t="inlineStr">
+      <c r="N12" s="6" t="inlineStr">
         <is>
           <t>Parent automation.git GitLab CI is mock</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="7" t="inlineStr">
+      <c r="A13" s="6" t="inlineStr">
         <is>
           <t>Jenkins</t>
         </is>
       </c>
-      <c r="B13" s="7" t="inlineStr">
+      <c r="B13" s="6" t="inlineStr">
         <is>
           <t>ASTRO-TB-REFRESH</t>
         </is>
       </c>
-      <c r="C13" s="7" t="inlineStr">
+      <c r="C13" s="6" t="inlineStr">
         <is>
           <t>astro-test-automation</t>
         </is>
       </c>
-      <c r="D13" s="7" t="inlineStr">
+      <c r="D13" s="6" t="inlineStr">
         <is>
           <t>Ant build.xml</t>
         </is>
       </c>
-      <c r="E13" s="7" t="inlineStr">
+      <c r="E13" s="6" t="inlineStr">
         <is>
           <t>Pre-regression</t>
         </is>
       </c>
-      <c r="F13" s="7" t="inlineStr">
+      <c r="F13" s="6" t="inlineStr">
         <is>
           <t>TB1</t>
         </is>
       </c>
-      <c r="G13" s="7" t="inlineStr">
+      <c r="G13" s="6" t="inlineStr">
         <is>
           <t>Testbed refresh</t>
         </is>
       </c>
-      <c r="H13" s="7" t="inlineStr">
+      <c r="H13" s="6" t="inlineStr">
         <is>
           <t>ASTRO</t>
         </is>
       </c>
-      <c r="I13" s="7" t="inlineStr">
+      <c r="I13" s="6" t="inlineStr">
         <is>
           <t>Logs</t>
         </is>
       </c>
-      <c r="J13" s="7" t="inlineStr">
+      <c r="J13" s="6" t="inlineStr">
         <is>
           <t>Unknown</t>
         </is>
       </c>
-      <c r="K13" s="7" t="inlineStr">
+      <c r="K13" s="6" t="inlineStr">
         <is>
           <t>Environment prep</t>
         </is>
       </c>
-      <c r="L13" s="7" t="inlineStr">
+      <c r="L13" s="6" t="inlineStr">
         <is>
           <t>astro/bin/build.xml</t>
         </is>
       </c>
-      <c r="M13" s="7" t="inlineStr">
+      <c r="M13" s="6" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="N13" s="7" t="inlineStr"/>
+      <c r="N13" s="6" t="inlineStr"/>
     </row>
     <row r="14">
-      <c r="A14" s="7" t="inlineStr">
+      <c r="A14" s="6" t="inlineStr">
         <is>
           <t>Jenkins</t>
         </is>
       </c>
-      <c r="B14" s="7" t="inlineStr">
+      <c r="B14" s="6" t="inlineStr">
         <is>
           <t>AGSUP_IDP_REGRESSION_SUITE</t>
         </is>
       </c>
-      <c r="C14" s="7" t="inlineStr">
+      <c r="C14" s="6" t="inlineStr">
         <is>
           <t>performance-test-automation</t>
         </is>
       </c>
-      <c r="D14" s="7" t="inlineStr">
+      <c r="D14" s="6" t="inlineStr">
         <is>
           <t>Build periodically</t>
         </is>
       </c>
-      <c r="E14" s="7" t="inlineStr">
+      <c r="E14" s="6" t="inlineStr">
         <is>
           <t>H 3 * * 1-5 (weekdays ~3 AM EDT)</t>
         </is>
       </c>
-      <c r="F14" s="7" t="inlineStr">
+      <c r="F14" s="6" t="inlineStr">
         <is>
           <t>Load servers</t>
         </is>
       </c>
-      <c r="G14" s="7" t="inlineStr">
+      <c r="G14" s="6" t="inlineStr">
         <is>
           <t>IDP Taurus YAML suite</t>
         </is>
       </c>
-      <c r="H14" s="7" t="inlineStr">
+      <c r="H14" s="6" t="inlineStr">
         <is>
           <t>Universal Platform IDP perf</t>
         </is>
       </c>
-      <c r="I14" s="7" t="inlineStr">
+      <c r="I14" s="6" t="inlineStr">
         <is>
           <t>Perf reports</t>
         </is>
       </c>
-      <c r="J14" s="7" t="inlineStr">
+      <c r="J14" s="6" t="inlineStr">
         <is>
           <t>Unknown</t>
         </is>
       </c>
-      <c r="K14" s="7" t="inlineStr">
+      <c r="K14" s="6" t="inlineStr">
         <is>
           <t>Scheduled regression (perf)</t>
         </is>
       </c>
-      <c r="L14" s="7" t="inlineStr">
+      <c r="L14" s="6" t="inlineStr">
         <is>
           <t>mobile2-api-db-validation/.../unite-msc-performance-testing-tracker.md</t>
         </is>
       </c>
-      <c r="M14" s="7" t="inlineStr">
+      <c r="M14" s="6" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="N14" s="7" t="inlineStr">
+      <c r="N14" s="6" t="inlineStr">
         <is>
           <t>Not functional API regression</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="7" t="inlineStr">
+      <c r="A15" s="6" t="inlineStr">
         <is>
           <t>Jenkins</t>
         </is>
       </c>
-      <c r="B15" s="7" t="inlineStr">
+      <c r="B15" s="6" t="inlineStr">
         <is>
           <t>AGSUP_UNITE_MSC_ENDURANCE</t>
         </is>
       </c>
-      <c r="C15" s="7" t="inlineStr">
+      <c r="C15" s="6" t="inlineStr">
         <is>
           <t>performance-test-automation</t>
         </is>
       </c>
-      <c r="D15" s="7" t="inlineStr">
+      <c r="D15" s="6" t="inlineStr">
         <is>
           <t>Manual parameterized</t>
         </is>
       </c>
-      <c r="E15" s="7" t="inlineStr">
+      <c r="E15" s="6" t="inlineStr">
         <is>
           <t>No periodic trigger (2026-07-02)</t>
         </is>
       </c>
-      <c r="F15" s="7" t="inlineStr">
+      <c r="F15" s="6" t="inlineStr">
         <is>
           <t>QC4 Stage1</t>
         </is>
       </c>
-      <c r="G15" s="7" t="inlineStr">
+      <c r="G15" s="6" t="inlineStr">
         <is>
           <t>unite-msc-non-idp-login-remote.yaml (+ choices)</t>
         </is>
       </c>
-      <c r="H15" s="7" t="inlineStr">
+      <c r="H15" s="6" t="inlineStr">
         <is>
           <t>Unite MSC perf</t>
         </is>
       </c>
-      <c r="I15" s="7" t="inlineStr">
+      <c r="I15" s="6" t="inlineStr">
         <is>
           <t>Optional artifacts</t>
         </is>
       </c>
-      <c r="J15" s="7" t="inlineStr">
+      <c r="J15" s="6" t="inlineStr">
         <is>
           <t>Unknown</t>
         </is>
       </c>
-      <c r="K15" s="7" t="inlineStr">
+      <c r="K15" s="6" t="inlineStr">
         <is>
           <t>Manual only</t>
         </is>
       </c>
-      <c r="L15" s="7" t="inlineStr">
+      <c r="L15" s="6" t="inlineStr">
         <is>
           <t>Same tracker doc</t>
         </is>
       </c>
-      <c r="M15" s="7" t="inlineStr">
+      <c r="M15" s="6" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="N15" s="7" t="inlineStr">
+      <c r="N15" s="6" t="inlineStr">
         <is>
           <t>IDP YAML exists; not default job choice</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="7" t="inlineStr">
+      <c r="A16" s="6" t="inlineStr">
         <is>
           <t>Jenkins</t>
         </is>
       </c>
-      <c r="B16" s="7" t="inlineStr">
+      <c r="B16" s="6" t="inlineStr">
         <is>
           <t>AGSUP_ENDURANCE_THROUGHPUT</t>
         </is>
       </c>
-      <c r="C16" s="7" t="inlineStr">
+      <c r="C16" s="6" t="inlineStr">
         <is>
           <t>performance-test-automation</t>
         </is>
       </c>
-      <c r="D16" s="7" t="inlineStr">
+      <c r="D16" s="6" t="inlineStr">
         <is>
           <t>Child of IDP suite</t>
         </is>
       </c>
-      <c r="E16" s="7" t="inlineStr">
+      <c r="E16" s="6" t="inlineStr">
         <is>
           <t>With IDP suite</t>
         </is>
       </c>
-      <c r="F16" s="7" t="inlineStr">
+      <c r="F16" s="6" t="inlineStr">
         <is>
           <t>Load servers</t>
         </is>
       </c>
-      <c r="G16" s="7" t="inlineStr">
+      <c r="G16" s="6" t="inlineStr">
         <is>
           <t>Parameterized YAML</t>
         </is>
       </c>
-      <c r="H16" s="7" t="inlineStr">
+      <c r="H16" s="6" t="inlineStr">
         <is>
           <t>UP perf throughput</t>
         </is>
       </c>
-      <c r="I16" s="7" t="inlineStr">
+      <c r="I16" s="6" t="inlineStr">
         <is>
           <t>Perf metrics</t>
         </is>
       </c>
-      <c r="J16" s="7" t="inlineStr">
+      <c r="J16" s="6" t="inlineStr">
         <is>
           <t>Unknown</t>
         </is>
       </c>
-      <c r="K16" s="7" t="inlineStr">
+      <c r="K16" s="6" t="inlineStr">
         <is>
           <t>Child job</t>
         </is>
       </c>
-      <c r="L16" s="7" t="inlineStr">
+      <c r="L16" s="6" t="inlineStr">
         <is>
           <t>Same tracker doc</t>
         </is>
       </c>
-      <c r="M16" s="7" t="inlineStr">
+      <c r="M16" s="6" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="N16" s="7" t="inlineStr"/>
+      <c r="N16" s="6" t="inlineStr"/>
     </row>
     <row r="17">
-      <c r="A17" s="7" t="inlineStr">
+      <c r="A17" s="6" t="inlineStr">
         <is>
           <t>Jenkins</t>
         </is>
       </c>
-      <c r="B17" s="7" t="inlineStr">
+      <c r="B17" s="6" t="inlineStr">
         <is>
           <t>V2/V3 UI regression (historical)</t>
         </is>
       </c>
-      <c r="C17" s="7" t="inlineStr">
+      <c r="C17" s="6" t="inlineStr">
         <is>
           <t>unite-test-automation / prime</t>
         </is>
       </c>
-      <c r="D17" s="7" t="inlineStr">
+      <c r="D17" s="6" t="inlineStr">
         <is>
           <t>Referenced in demand planning imports</t>
         </is>
       </c>
-      <c r="E17" s="7" t="inlineStr">
+      <c r="E17" s="6" t="inlineStr">
         <is>
           <t>TBD</t>
         </is>
       </c>
-      <c r="F17" s="7" t="inlineStr">
+      <c r="F17" s="6" t="inlineStr">
         <is>
           <t>TBD</t>
         </is>
       </c>
-      <c r="G17" s="7" t="inlineStr">
+      <c r="G17" s="6" t="inlineStr">
         <is>
           <t>TBD</t>
         </is>
       </c>
-      <c r="H17" s="7" t="inlineStr">
+      <c r="H17" s="6" t="inlineStr">
         <is>
           <t>~779+ combined TCs Apr 2026 claim</t>
         </is>
       </c>
-      <c r="I17" s="7" t="inlineStr">
+      <c r="I17" s="6" t="inlineStr">
         <is>
           <t>HTML reports</t>
         </is>
       </c>
-      <c r="J17" s="7" t="inlineStr">
+      <c r="J17" s="6" t="inlineStr">
         <is>
           <t>TBD</t>
         </is>
       </c>
-      <c r="K17" s="7" t="inlineStr">
+      <c r="K17" s="6" t="inlineStr">
         <is>
           <t>TBD — refresh required</t>
         </is>
       </c>
-      <c r="L17" s="7" t="inlineStr">
+      <c r="L17" s="6" t="inlineStr">
         <is>
           <t>10_IMPORTS_RAW/confluence_exports/Demand Planning Reports/</t>
         </is>
       </c>
-      <c r="M17" s="7" t="inlineStr">
+      <c r="M17" s="6" t="inlineStr">
         <is>
           <t>Low</t>
         </is>
       </c>
-      <c r="N17" s="7" t="inlineStr">
+      <c r="N17" s="6" t="inlineStr">
         <is>
           <t>Historical counts; not verified current</t>
         </is>
@@ -4412,132 +4520,132 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="8" t="inlineStr">
+      <c r="A2" s="7" t="inlineStr">
         <is>
           <t>CL-003</t>
         </is>
       </c>
-      <c r="B2" s="8" t="inlineStr">
+      <c r="B2" s="7" t="inlineStr">
         <is>
           <t>Mobile 2 100% (24/24)</t>
         </is>
       </c>
-      <c r="C2" s="8" t="inlineStr">
+      <c r="C2" s="7" t="inlineStr">
         <is>
           <t>Rejected</t>
         </is>
       </c>
-      <c r="D2" s="8" t="inlineStr">
+      <c r="D2" s="7" t="inlineStr">
         <is>
           <t>Replaced — see CL-004 CL-005</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="9" t="inlineStr">
+      <c r="A3" s="8" t="inlineStr">
         <is>
           <t>CL-005</t>
         </is>
       </c>
-      <c r="B3" s="9" t="inlineStr">
+      <c r="B3" s="8" t="inlineStr">
         <is>
           <t>Mobile 2 projected 96% (24/25) pending sign-off</t>
         </is>
       </c>
-      <c r="C3" s="9" t="inlineStr">
+      <c r="C3" s="8" t="inlineStr">
         <is>
           <t>Pending verification</t>
         </is>
       </c>
-      <c r="D3" s="9" t="inlineStr">
+      <c r="D3" s="8" t="inlineStr">
         <is>
           <t>QC4/Stage1 rerun + matrix refresh</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="8" t="inlineStr">
+      <c r="A4" s="7" t="inlineStr">
         <is>
           <t>CL-006</t>
         </is>
       </c>
-      <c r="B4" s="8" t="inlineStr">
+      <c r="B4" s="7" t="inlineStr">
         <is>
           <t>Mobile 1 22.2% verified</t>
         </is>
       </c>
-      <c r="C4" s="8" t="inlineStr">
+      <c r="C4" s="7" t="inlineStr">
         <is>
           <t>Rejected</t>
         </is>
       </c>
-      <c r="D4" s="8" t="inlineStr">
+      <c r="D4" s="7" t="inlineStr">
         <is>
           <t>Split verified vs pending</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="9" t="inlineStr">
+      <c r="A5" s="8" t="inlineStr">
         <is>
           <t>CL-008</t>
         </is>
       </c>
-      <c r="B5" s="9" t="inlineStr">
+      <c r="B5" s="8" t="inlineStr">
         <is>
           <t>Mobile 1 implemented 6/27 pending evidence</t>
         </is>
       </c>
-      <c r="C5" s="9" t="inlineStr">
+      <c r="C5" s="8" t="inlineStr">
         <is>
           <t>Pending verification</t>
         </is>
       </c>
-      <c r="D5" s="9" t="inlineStr">
+      <c r="D5" s="8" t="inlineStr">
         <is>
           <t>Sprint evidence + workbook mapping</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="8" t="inlineStr">
+      <c r="A6" s="7" t="inlineStr">
         <is>
           <t>CL-009</t>
         </is>
       </c>
-      <c r="B6" s="8" t="inlineStr">
+      <c r="B6" s="7" t="inlineStr">
         <is>
           <t>GitHub Actions not implemented</t>
         </is>
       </c>
-      <c r="C6" s="8" t="inlineStr">
+      <c r="C6" s="7" t="inlineStr">
         <is>
           <t>Rejected</t>
         </is>
       </c>
-      <c r="D6" s="8" t="inlineStr">
+      <c r="D6" s="7" t="inlineStr">
         <is>
           <t>Externally validated Dashboard slice</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="8" t="inlineStr">
+      <c r="A7" s="7" t="inlineStr">
         <is>
           <t>CL-011</t>
         </is>
       </c>
-      <c r="B7" s="8" t="inlineStr">
+      <c r="B7" s="7" t="inlineStr">
         <is>
           <t>V3 GitLab hard merge gate</t>
         </is>
       </c>
-      <c r="C7" s="8" t="inlineStr">
+      <c r="C7" s="7" t="inlineStr">
         <is>
           <t>Rejected</t>
         </is>
       </c>
-      <c r="D7" s="8" t="inlineStr">
+      <c r="D7" s="7" t="inlineStr">
         <is>
           <t>Reclassify scheduled hard-fail</t>
         </is>

</xml_diff>

<commit_message>
Add new assessments and coverage summaries for Government Savings automation
- Introduced detailed assessments for ASTRO/SFRP and Back-office/Batch automation, outlining current status, execution findings, and revalidation efforts required.
- Added new CSV files for business coverage metrics, including the Government Savings Business Coverage Register and Legacy Unite Module Status.
- Updated the Government Savings Automation Coverage Assessment document to reflect the latest findings and recommendations for operational activation.
- Created a comprehensive Business Coverage Summary to provide leadership with insights into automation maturity across platforms.

These additions aim to enhance visibility into automation coverage and facilitate informed decision-making for future improvements.
</commit_message>
<xml_diff>
--- a/government-savings-automation-assessment/03-analysis/government-savings-coverage-matrix.xlsx
+++ b/government-savings-automation-assessment/03-analysis/government-savings-coverage-matrix.xlsx
@@ -8,12 +8,13 @@
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Executive Summary" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Coverage Matrix" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CI Jobs Gates" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Unresolved Verification" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Business Coverage" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Coverage Matrix" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CI Jobs Gates" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Unresolved Verification" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Coverage Matrix'!$A$1:$U$21</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Coverage Matrix'!$A$1:$U$21</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -961,6 +962,2194 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:O29"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="24" customWidth="1" min="1" max="1"/>
+    <col width="39" customWidth="1" min="2" max="2"/>
+    <col width="47" customWidth="1" min="3" max="3"/>
+    <col width="11" customWidth="1" min="4" max="4"/>
+    <col width="13" customWidth="1" min="5" max="5"/>
+    <col width="28" customWidth="1" min="6" max="6"/>
+    <col width="48" customWidth="1" min="7" max="7"/>
+    <col width="47" customWidth="1" min="8" max="8"/>
+    <col width="48" customWidth="1" min="9" max="9"/>
+    <col width="44" customWidth="1" min="10" max="10"/>
+    <col width="48" customWidth="1" min="11" max="11"/>
+    <col width="12" customWidth="1" min="12" max="12"/>
+    <col width="48" customWidth="1" min="13" max="13"/>
+    <col width="12" customWidth="1" min="14" max="14"/>
+    <col width="48" customWidth="1" min="15" max="15"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="2" t="inlineStr">
+        <is>
+          <t>business_area</t>
+        </is>
+      </c>
+      <c r="B1" s="2" t="inlineStr">
+        <is>
+          <t>sub_area</t>
+        </is>
+      </c>
+      <c r="C1" s="2" t="inlineStr">
+        <is>
+          <t>metric_label</t>
+        </is>
+      </c>
+      <c r="D1" s="2" t="inlineStr">
+        <is>
+          <t>numerator</t>
+        </is>
+      </c>
+      <c r="E1" s="2" t="inlineStr">
+        <is>
+          <t>denominator</t>
+        </is>
+      </c>
+      <c r="F1" s="2" t="inlineStr">
+        <is>
+          <t>counting_unit</t>
+        </is>
+      </c>
+      <c r="G1" s="2" t="inlineStr">
+        <is>
+          <t>percent_class</t>
+        </is>
+      </c>
+      <c r="H1" s="2" t="inlineStr">
+        <is>
+          <t>implementation_status</t>
+        </is>
+      </c>
+      <c r="I1" s="2" t="inlineStr">
+        <is>
+          <t>execution_status</t>
+        </is>
+      </c>
+      <c r="J1" s="2" t="inlineStr">
+        <is>
+          <t>scheduled_status</t>
+        </is>
+      </c>
+      <c r="K1" s="2" t="inlineStr">
+        <is>
+          <t>leadership_safe_wording</t>
+        </is>
+      </c>
+      <c r="L1" s="2" t="inlineStr">
+        <is>
+          <t>confidence</t>
+        </is>
+      </c>
+      <c r="M1" s="2" t="inlineStr">
+        <is>
+          <t>evidence_path</t>
+        </is>
+      </c>
+      <c r="N1" s="2" t="inlineStr">
+        <is>
+          <t>as_of_date</t>
+        </is>
+      </c>
+      <c r="O1" s="2" t="inlineStr">
+        <is>
+          <t>notes</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="6" t="inlineStr">
+        <is>
+          <t>Unite MSC</t>
+        </is>
+      </c>
+      <c r="B2" s="6" t="inlineStr">
+        <is>
+          <t>Mobile 2 API</t>
+        </is>
+      </c>
+      <c r="C2" s="6" t="inlineStr">
+        <is>
+          <t>Automatable business endpoints implemented</t>
+        </is>
+      </c>
+      <c r="D2" s="6" t="inlineStr">
+        <is>
+          <t>24</t>
+        </is>
+      </c>
+      <c r="E2" s="6" t="inlineStr">
+        <is>
+          <t>24</t>
+        </is>
+      </c>
+      <c r="F2" s="6" t="inlineStr">
+        <is>
+          <t>business API endpoints</t>
+        </is>
+      </c>
+      <c r="G2" s="6" t="inlineStr">
+        <is>
+          <t>Verified from current denominator and repository evidence</t>
+        </is>
+      </c>
+      <c r="H2" s="6" t="inlineStr">
+        <is>
+          <t>Complete for automatable scope</t>
+        </is>
+      </c>
+      <c r="I2" s="6" t="inlineStr">
+        <is>
+          <t>Stale master run 22/25 (2026-07-14); 2 endpoints added post-sign-off</t>
+        </is>
+      </c>
+      <c r="J2" s="6" t="inlineStr">
+        <is>
+          <t>Not scheduled — QA-1405 pending</t>
+        </is>
+      </c>
+      <c r="K2" s="6" t="inlineStr">
+        <is>
+          <t>Mobile 2 automation is complete for the currently defined automatable business scope; destructive operations intentionally in smoke/module suites; recurring GitLab execution remains follow-up</t>
+        </is>
+      </c>
+      <c r="L2" s="6" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="M2" s="6" t="inlineStr">
+        <is>
+          <t>mobile2-endpoint-current-state.csv @ cee0de9</t>
+        </is>
+      </c>
+      <c r="N2" s="6" t="inlineStr">
+        <is>
+          <t>2026-07-21</t>
+        </is>
+      </c>
+      <c r="O2" s="6" t="inlineStr">
+        <is>
+          <t>Excludes mobilemembers harness endpoint from automatable scope</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="6" t="inlineStr">
+        <is>
+          <t>Unite MSC</t>
+        </is>
+      </c>
+      <c r="B3" s="6" t="inlineStr">
+        <is>
+          <t>Mobile 2 API</t>
+        </is>
+      </c>
+      <c r="C3" s="6" t="inlineStr">
+        <is>
+          <t>Documented business endpoints (incl. harness)</t>
+        </is>
+      </c>
+      <c r="D3" s="6" t="inlineStr">
+        <is>
+          <t>24</t>
+        </is>
+      </c>
+      <c r="E3" s="6" t="inlineStr">
+        <is>
+          <t>25</t>
+        </is>
+      </c>
+      <c r="F3" s="6" t="inlineStr">
+        <is>
+          <t>business API endpoints</t>
+        </is>
+      </c>
+      <c r="G3" s="6" t="inlineStr">
+        <is>
+          <t>Verified implementation estimate</t>
+        </is>
+      </c>
+      <c r="H3" s="6" t="inlineStr">
+        <is>
+          <t>24/25 implemented</t>
+        </is>
+      </c>
+      <c r="I3" s="6" t="inlineStr">
+        <is>
+          <t>Stale execution 88%</t>
+        </is>
+      </c>
+      <c r="J3" s="6" t="inlineStr">
+        <is>
+          <t>Not scheduled</t>
+        </is>
+      </c>
+      <c r="K3" s="6" t="inlineStr">
+        <is>
+          <t>Near-complete for documented business scope; harness endpoint excluded from automation numerator by design</t>
+        </is>
+      </c>
+      <c r="L3" s="6" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="M3" s="6" t="inlineStr">
+        <is>
+          <t>mobile2-endpoint-current-state.csv</t>
+        </is>
+      </c>
+      <c r="N3" s="6" t="inlineStr">
+        <is>
+          <t>2026-07-21</t>
+        </is>
+      </c>
+      <c r="O3" s="6" t="inlineStr"/>
+    </row>
+    <row r="4">
+      <c r="A4" s="6" t="inlineStr">
+        <is>
+          <t>Unite MSC</t>
+        </is>
+      </c>
+      <c r="B4" s="6" t="inlineStr">
+        <is>
+          <t>Mobile 1 API</t>
+        </is>
+      </c>
+      <c r="C4" s="6" t="inlineStr">
+        <is>
+          <t>Documented business endpoints</t>
+        </is>
+      </c>
+      <c r="D4" s="6" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="E4" s="6" t="inlineStr">
+        <is>
+          <t>27</t>
+        </is>
+      </c>
+      <c r="F4" s="6" t="inlineStr">
+        <is>
+          <t>business API endpoints</t>
+        </is>
+      </c>
+      <c r="G4" s="6" t="inlineStr">
+        <is>
+          <t>Verified from current denominator and repository evidence</t>
+        </is>
+      </c>
+      <c r="H4" s="6" t="inlineStr">
+        <is>
+          <t>Partial — sprint expansion</t>
+        </is>
+      </c>
+      <c r="I4" s="6" t="inlineStr">
+        <is>
+          <t>1/27 execution-verified (session)</t>
+        </is>
+      </c>
+      <c r="J4" s="6" t="inlineStr">
+        <is>
+          <t>Not scheduled</t>
+        </is>
+      </c>
+      <c r="K4" s="6" t="inlineStr">
+        <is>
+          <t>Partial coverage with expansion in progress on owner profile beneficiary and bank routing</t>
+        </is>
+      </c>
+      <c r="L4" s="6" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="M4" s="6" t="inlineStr">
+        <is>
+          <t>mobile1-endpoint-current-state.csv @ cee0de9</t>
+        </is>
+      </c>
+      <c r="N4" s="6" t="inlineStr">
+        <is>
+          <t>2026-07-21</t>
+        </is>
+      </c>
+      <c r="O4" s="6" t="inlineStr"/>
+    </row>
+    <row r="5">
+      <c r="A5" s="6" t="inlineStr">
+        <is>
+          <t>Unite MSC</t>
+        </is>
+      </c>
+      <c r="B5" s="6" t="inlineStr">
+        <is>
+          <t>Mobile Enrollment API</t>
+        </is>
+      </c>
+      <c r="C5" s="6" t="inlineStr">
+        <is>
+          <t>Bootstrap / pilot endpoints</t>
+        </is>
+      </c>
+      <c r="D5" s="6" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="E5" s="6" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="F5" s="6" t="inlineStr">
+        <is>
+          <t>business API endpoints</t>
+        </is>
+      </c>
+      <c r="G5" s="6" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="H5" s="6" t="inlineStr">
+        <is>
+          <t>Bootstrap smoke only</t>
+        </is>
+      </c>
+      <c r="I5" s="6" t="inlineStr">
+        <is>
+          <t>No execution evidence</t>
+        </is>
+      </c>
+      <c r="J5" s="6" t="inlineStr">
+        <is>
+          <t>Not scheduled</t>
+        </is>
+      </c>
+      <c r="K5" s="6" t="inlineStr">
+        <is>
+          <t>Pilot framework in place; endpoint inventory and automation scope not yet enumerated</t>
+        </is>
+      </c>
+      <c r="L5" s="6" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="M5" s="6" t="inlineStr">
+        <is>
+          <t>mobile/enrollment/ @ cee0de9</t>
+        </is>
+      </c>
+      <c r="N5" s="6" t="inlineStr">
+        <is>
+          <t>2026-07-21</t>
+        </is>
+      </c>
+      <c r="O5" s="6" t="inlineStr">
+        <is>
+          <t>Do not include in MSC combined %</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="6" t="inlineStr">
+        <is>
+          <t>Unite MSC</t>
+        </is>
+      </c>
+      <c r="B6" s="6" t="inlineStr">
+        <is>
+          <t>UniteMSC microservices</t>
+        </is>
+      </c>
+      <c r="C6" s="6" t="inlineStr">
+        <is>
+          <t>Service BDD features (aggregate)</t>
+        </is>
+      </c>
+      <c r="D6" s="6" t="inlineStr">
+        <is>
+          <t>112</t>
+        </is>
+      </c>
+      <c r="E6" s="6" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="F6" s="6" t="inlineStr">
+        <is>
+          <t>Cucumber features</t>
+        </is>
+      </c>
+      <c r="G6" s="6" t="inlineStr">
+        <is>
+          <t>Program estimate requiring reconciliation</t>
+        </is>
+      </c>
+      <c r="H6" s="6" t="inlineStr">
+        <is>
+          <t>Substantial service-level assets</t>
+        </is>
+      </c>
+      <c r="I6" s="6" t="inlineStr">
+        <is>
+          <t>Service CI only</t>
+        </is>
+      </c>
+      <c r="J6" s="6" t="inlineStr">
+        <is>
+          <t>Per-repo GitLab pipeline</t>
+        </is>
+      </c>
+      <c r="K6" s="6" t="inlineStr">
+        <is>
+          <t>Service acceptance automation exists; not a substitute for BFF API regression</t>
+        </is>
+      </c>
+      <c r="L6" s="6" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="M6" s="6" t="inlineStr">
+        <is>
+          <t>UniteMSC repos / unite-mobile2 features</t>
+        </is>
+      </c>
+      <c r="N6" s="6" t="inlineStr">
+        <is>
+          <t>2026-07-21</t>
+        </is>
+      </c>
+      <c r="O6" s="6" t="inlineStr"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="6" t="inlineStr">
+        <is>
+          <t>Unite MSC</t>
+        </is>
+      </c>
+      <c r="B7" s="6" t="inlineStr">
+        <is>
+          <t>Application source code</t>
+        </is>
+      </c>
+      <c r="C7" s="6" t="inlineStr">
+        <is>
+          <t>JaCoCo on service repos</t>
+        </is>
+      </c>
+      <c r="D7" s="6" t="inlineStr">
+        <is>
+          <t>13</t>
+        </is>
+      </c>
+      <c r="E7" s="6" t="inlineStr">
+        <is>
+          <t>13</t>
+        </is>
+      </c>
+      <c r="F7" s="6" t="inlineStr">
+        <is>
+          <t>Java microservice repos</t>
+        </is>
+      </c>
+      <c r="G7" s="6" t="inlineStr">
+        <is>
+          <t>Verified from repository code</t>
+        </is>
+      </c>
+      <c r="H7" s="6" t="inlineStr">
+        <is>
+          <t>Generated in CI</t>
+        </is>
+      </c>
+      <c r="I7" s="6" t="inlineStr">
+        <is>
+          <t>Sonar disabled</t>
+        </is>
+      </c>
+      <c r="J7" s="6" t="inlineStr">
+        <is>
+          <t>Service build/test gate</t>
+        </is>
+      </c>
+      <c r="K7" s="6" t="inlineStr">
+        <is>
+          <t>Application line coverage separate from business automation; no coverage-delta MR gate</t>
+        </is>
+      </c>
+      <c r="L7" s="6" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="M7" s="6" t="inlineStr">
+        <is>
+          <t>source-code-coverage-assessment.md</t>
+        </is>
+      </c>
+      <c r="N7" s="6" t="inlineStr">
+        <is>
+          <t>2026-07-21</t>
+        </is>
+      </c>
+      <c r="O7" s="6" t="inlineStr"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="6" t="inlineStr">
+        <is>
+          <t>Unite MSC</t>
+        </is>
+      </c>
+      <c r="B8" s="6" t="inlineStr">
+        <is>
+          <t>GitHub Actions</t>
+        </is>
+      </c>
+      <c r="C8" s="6" t="inlineStr">
+        <is>
+          <t>Mobile 2 Dashboard deployment validation</t>
+        </is>
+      </c>
+      <c r="D8" s="6" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="E8" s="6" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="F8" s="6" t="inlineStr">
+        <is>
+          <t>validated vertical slice</t>
+        </is>
+      </c>
+      <c r="G8" s="6" t="inlineStr">
+        <is>
+          <t>Verified external</t>
+        </is>
+      </c>
+      <c r="H8" s="6" t="inlineStr">
+        <is>
+          <t>Deployment slice validated</t>
+        </is>
+      </c>
+      <c r="I8" s="6" t="inlineStr">
+        <is>
+          <t>Externally validated</t>
+        </is>
+      </c>
+      <c r="J8" s="6" t="inlineStr">
+        <is>
+          <t>Workflow not in clone</t>
+        </is>
+      </c>
+      <c r="K8" s="6" t="inlineStr">
+        <is>
+          <t>Deployment validation — not nightly business regression</t>
+        </is>
+      </c>
+      <c r="L8" s="6" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="M8" s="6" t="inlineStr">
+        <is>
+          <t>17-MOBILE2-NEXUS-GITHUB-ACTIONS-PIPELINE.md</t>
+        </is>
+      </c>
+      <c r="N8" s="6" t="inlineStr">
+        <is>
+          <t>2026-07-21</t>
+        </is>
+      </c>
+      <c r="O8" s="6" t="inlineStr"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="6" t="inlineStr">
+        <is>
+          <t>Universal Platform</t>
+        </is>
+      </c>
+      <c r="B9" s="6" t="inlineStr">
+        <is>
+          <t>Universal Enrollment</t>
+        </is>
+      </c>
+      <c r="C9" s="6" t="inlineStr">
+        <is>
+          <t>TestNG methods in nightly inventory</t>
+        </is>
+      </c>
+      <c r="D9" s="6" t="inlineStr">
+        <is>
+          <t>303</t>
+        </is>
+      </c>
+      <c r="E9" s="6" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="F9" s="6" t="inlineStr">
+        <is>
+          <t>TestNG test methods</t>
+        </is>
+      </c>
+      <c r="G9" s="6" t="inlineStr">
+        <is>
+          <t>Verified count — no business % denominator</t>
+        </is>
+      </c>
+      <c r="H9" s="6" t="inlineStr">
+        <is>
+          <t>Near-complete for approved regression scope</t>
+        </is>
+      </c>
+      <c r="I9" s="6" t="inlineStr">
+        <is>
+          <t>Active in GitLab nightly</t>
+        </is>
+      </c>
+      <c r="J9" s="6" t="inlineStr">
+        <is>
+          <t>scheduled_regression_job</t>
+        </is>
+      </c>
+      <c r="K9" s="6" t="inlineStr">
+        <is>
+          <t>Majority of current high-priority enrollment journeys automated in Modern Unite nightly</t>
+        </is>
+      </c>
+      <c r="L9" s="6" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="M9" s="6" t="inlineStr">
+        <is>
+          <t>universal-platform-coverage/01-analysis/csv/final-workstream-summary.csv</t>
+        </is>
+      </c>
+      <c r="N9" s="6" t="inlineStr">
+        <is>
+          <t>2026-07-01</t>
+        </is>
+      </c>
+      <c r="O9" s="6" t="inlineStr">
+        <is>
+          <t>Do not state 95% without approved denominator</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="6" t="inlineStr">
+        <is>
+          <t>Universal Platform</t>
+        </is>
+      </c>
+      <c r="B10" s="6" t="inlineStr">
+        <is>
+          <t>IDP / Authentication</t>
+        </is>
+      </c>
+      <c r="C10" s="6" t="inlineStr">
+        <is>
+          <t>TestNG methods in nightly inventory</t>
+        </is>
+      </c>
+      <c r="D10" s="6" t="inlineStr">
+        <is>
+          <t>56</t>
+        </is>
+      </c>
+      <c r="E10" s="6" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="F10" s="6" t="inlineStr">
+        <is>
+          <t>TestNG test methods</t>
+        </is>
+      </c>
+      <c r="G10" s="6" t="inlineStr">
+        <is>
+          <t>Verified count — no business % denominator</t>
+        </is>
+      </c>
+      <c r="H10" s="6" t="inlineStr">
+        <is>
+          <t>Near-complete for approved regression scope</t>
+        </is>
+      </c>
+      <c r="I10" s="6" t="inlineStr">
+        <is>
+          <t>Active in GitLab nightly</t>
+        </is>
+      </c>
+      <c r="J10" s="6" t="inlineStr">
+        <is>
+          <t>scheduled_regression_job</t>
+        </is>
+      </c>
+      <c r="K10" s="6" t="inlineStr">
+        <is>
+          <t>Near-complete automation for current documented IDP regression scope</t>
+        </is>
+      </c>
+      <c r="L10" s="6" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="M10" s="6" t="inlineStr">
+        <is>
+          <t>final-workstream-summary.csv</t>
+        </is>
+      </c>
+      <c r="N10" s="6" t="inlineStr">
+        <is>
+          <t>2026-07-01</t>
+        </is>
+      </c>
+      <c r="O10" s="6" t="inlineStr"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="6" t="inlineStr">
+        <is>
+          <t>Universal Platform</t>
+        </is>
+      </c>
+      <c r="B11" s="6" t="inlineStr">
+        <is>
+          <t>Withdrawals</t>
+        </is>
+      </c>
+      <c r="C11" s="6" t="inlineStr">
+        <is>
+          <t>TestNG methods in nightly inventory</t>
+        </is>
+      </c>
+      <c r="D11" s="6" t="inlineStr">
+        <is>
+          <t>20</t>
+        </is>
+      </c>
+      <c r="E11" s="6" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="F11" s="6" t="inlineStr">
+        <is>
+          <t>TestNG test methods</t>
+        </is>
+      </c>
+      <c r="G11" s="6" t="inlineStr">
+        <is>
+          <t>Verified count</t>
+        </is>
+      </c>
+      <c r="H11" s="6" t="inlineStr">
+        <is>
+          <t>Near-complete for withdrawal regression scope</t>
+        </is>
+      </c>
+      <c r="I11" s="6" t="inlineStr">
+        <is>
+          <t>Active in GitLab nightly</t>
+        </is>
+      </c>
+      <c r="J11" s="6" t="inlineStr">
+        <is>
+          <t>scheduled_regression_job</t>
+        </is>
+      </c>
+      <c r="K11" s="6" t="inlineStr">
+        <is>
+          <t>Withdrawal domain automated in nightly; transfers adjacent (12 V2 methods)</t>
+        </is>
+      </c>
+      <c r="L11" s="6" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="M11" s="6" t="inlineStr">
+        <is>
+          <t>final-workstream-summary.csv</t>
+        </is>
+      </c>
+      <c r="N11" s="6" t="inlineStr">
+        <is>
+          <t>2026-07-01</t>
+        </is>
+      </c>
+      <c r="O11" s="6" t="inlineStr"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="6" t="inlineStr">
+        <is>
+          <t>Universal Platform</t>
+        </is>
+      </c>
+      <c r="B12" s="6" t="inlineStr">
+        <is>
+          <t>Entity / ABLE Entity</t>
+        </is>
+      </c>
+      <c r="C12" s="6" t="inlineStr">
+        <is>
+          <t>Implemented scenarios</t>
+        </is>
+      </c>
+      <c r="D12" s="6" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="E12" s="6" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="F12" s="6" t="inlineStr">
+        <is>
+          <t>business scenarios</t>
+        </is>
+      </c>
+      <c r="G12" s="6" t="inlineStr">
+        <is>
+          <t>Verified implementation estimate</t>
+        </is>
+      </c>
+      <c r="H12" s="6" t="inlineStr">
+        <is>
+          <t>Partial — 6 scenarios in repo</t>
+        </is>
+      </c>
+      <c r="I12" s="6" t="inlineStr">
+        <is>
+          <t>Not confirmed in nightly job</t>
+        </is>
+      </c>
+      <c r="J12" s="6" t="inlineStr">
+        <is>
+          <t>Unknown pipeline inclusion</t>
+        </is>
+      </c>
+      <c r="K12" s="6" t="inlineStr">
+        <is>
+          <t>Partial coverage with expansion in progress; remaining work primarily Entity and newly migrated features</t>
+        </is>
+      </c>
+      <c r="L12" s="6" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="M12" s="6" t="inlineStr">
+        <is>
+          <t>prime-test-automation/unite/unite-entity/</t>
+        </is>
+      </c>
+      <c r="N12" s="6" t="inlineStr">
+        <is>
+          <t>2026-07-01</t>
+        </is>
+      </c>
+      <c r="O12" s="6" t="inlineStr">
+        <is>
+          <t>Do not state 25% without denominator</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="6" t="inlineStr">
+        <is>
+          <t>Universal Platform</t>
+        </is>
+      </c>
+      <c r="B13" s="6" t="inlineStr">
+        <is>
+          <t>Angular lib-ui</t>
+        </is>
+      </c>
+      <c r="C13" s="6" t="inlineStr">
+        <is>
+          <t>Component tests</t>
+        </is>
+      </c>
+      <c r="D13" s="6" t="inlineStr">
+        <is>
+          <t>22</t>
+        </is>
+      </c>
+      <c r="E13" s="6" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="F13" s="6" t="inlineStr">
+        <is>
+          <t>component tests</t>
+        </is>
+      </c>
+      <c r="G13" s="6" t="inlineStr">
+        <is>
+          <t>Verified count</t>
+        </is>
+      </c>
+      <c r="H13" s="6" t="inlineStr">
+        <is>
+          <t>Component-level only</t>
+        </is>
+      </c>
+      <c r="I13" s="6" t="inlineStr">
+        <is>
+          <t>Manual/CI on push</t>
+        </is>
+      </c>
+      <c r="J13" s="6" t="inlineStr">
+        <is>
+          <t>accountowner_build_tdd partial</t>
+        </is>
+      </c>
+      <c r="K13" s="6" t="inlineStr">
+        <is>
+          <t>Component tests — not E2E business journey coverage</t>
+        </is>
+      </c>
+      <c r="L13" s="6" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="M13" s="6" t="inlineStr">
+        <is>
+          <t>universal-platform-coverage/01-analysis/07-angular-analysis.md</t>
+        </is>
+      </c>
+      <c r="N13" s="6" t="inlineStr">
+        <is>
+          <t>2026-07-01</t>
+        </is>
+      </c>
+      <c r="O13" s="6" t="inlineStr"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="6" t="inlineStr">
+        <is>
+          <t>Universal Platform</t>
+        </is>
+      </c>
+      <c r="B14" s="6" t="inlineStr">
+        <is>
+          <t>Universal API (scoped)</t>
+        </is>
+      </c>
+      <c r="C14" s="6" t="inlineStr">
+        <is>
+          <t>Unique HTTP operations</t>
+        </is>
+      </c>
+      <c r="D14" s="6" t="inlineStr">
+        <is>
+          <t>11</t>
+        </is>
+      </c>
+      <c r="E14" s="6" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="F14" s="6" t="inlineStr">
+        <is>
+          <t>API operations</t>
+        </is>
+      </c>
+      <c r="G14" s="6" t="inlineStr">
+        <is>
+          <t>Verified count — partial scheduling</t>
+        </is>
+      </c>
+      <c r="H14" s="6" t="inlineStr">
+        <is>
+          <t>11 ops mapped in UP ledger</t>
+        </is>
+      </c>
+      <c r="I14" s="6" t="inlineStr">
+        <is>
+          <t>Metadataweb scheduled only</t>
+        </is>
+      </c>
+      <c r="J14" s="6" t="inlineStr">
+        <is>
+          <t>scheduled_metadataweb_stage1</t>
+        </is>
+      </c>
+      <c r="K14" s="6" t="inlineStr">
+        <is>
+          <t>API automation exists beyond metadata; only metadataweb on GitLab schedule today</t>
+        </is>
+      </c>
+      <c r="L14" s="6" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="M14" s="6" t="inlineStr">
+        <is>
+          <t>api-operation-mapping.csv</t>
+        </is>
+      </c>
+      <c r="N14" s="6" t="inlineStr">
+        <is>
+          <t>2026-07-01</t>
+        </is>
+      </c>
+      <c r="O14" s="6" t="inlineStr"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="6" t="inlineStr">
+        <is>
+          <t>Universal Platform</t>
+        </is>
+      </c>
+      <c r="B15" s="6" t="inlineStr">
+        <is>
+          <t>Performance journeys</t>
+        </is>
+      </c>
+      <c r="C15" s="6" t="inlineStr">
+        <is>
+          <t>In-scope JMeter journeys</t>
+        </is>
+      </c>
+      <c r="D15" s="6" t="inlineStr">
+        <is>
+          <t>15</t>
+        </is>
+      </c>
+      <c r="E15" s="6" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="F15" s="6" t="inlineStr">
+        <is>
+          <t>business journeys</t>
+        </is>
+      </c>
+      <c r="G15" s="6" t="inlineStr">
+        <is>
+          <t>Verified count</t>
+        </is>
+      </c>
+      <c r="H15" s="6" t="inlineStr">
+        <is>
+          <t>IDP perf scheduled; others manual</t>
+        </is>
+      </c>
+      <c r="I15" s="6" t="inlineStr">
+        <is>
+          <t>AGSUP_IDP_REGRESSION_SUITE weekdays</t>
+        </is>
+      </c>
+      <c r="J15" s="6" t="inlineStr">
+        <is>
+          <t>Partial scheduled</t>
+        </is>
+      </c>
+      <c r="K15" s="6" t="inlineStr">
+        <is>
+          <t>Performance assets exist; not all journeys on recurring schedule</t>
+        </is>
+      </c>
+      <c r="L15" s="6" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="M15" s="6" t="inlineStr">
+        <is>
+          <t>performance-journey-mapping.csv</t>
+        </is>
+      </c>
+      <c r="N15" s="6" t="inlineStr">
+        <is>
+          <t>2026-07-01</t>
+        </is>
+      </c>
+      <c r="O15" s="6" t="inlineStr"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="6" t="inlineStr">
+        <is>
+          <t>Universal Platform</t>
+        </is>
+      </c>
+      <c r="B16" s="6" t="inlineStr">
+        <is>
+          <t>Nightly inventory share (technical)</t>
+        </is>
+      </c>
+      <c r="C16" s="6" t="inlineStr">
+        <is>
+          <t>Scoped TestNG methods</t>
+        </is>
+      </c>
+      <c r="D16" s="6" t="inlineStr">
+        <is>
+          <t>379</t>
+        </is>
+      </c>
+      <c r="E16" s="6" t="inlineStr">
+        <is>
+          <t>436</t>
+        </is>
+      </c>
+      <c r="F16" s="6" t="inlineStr">
+        <is>
+          <t>TestNG methods</t>
+        </is>
+      </c>
+      <c r="G16" s="6" t="inlineStr">
+        <is>
+          <t>Verified inventory share only</t>
+        </is>
+      </c>
+      <c r="H16" s="6" t="inlineStr">
+        <is>
+          <t>Implementation in repo</t>
+        </is>
+      </c>
+      <c r="I16" s="6" t="inlineStr">
+        <is>
+          <t>Active GitLab nightly</t>
+        </is>
+      </c>
+      <c r="J16" s="6" t="inlineStr">
+        <is>
+          <t>scheduled_regression_job</t>
+        </is>
+      </c>
+      <c r="K16" s="6" t="inlineStr">
+        <is>
+          <t>Technical appendix only — inventory share not functional completeness</t>
+        </is>
+      </c>
+      <c r="L16" s="6" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="M16" s="6" t="inlineStr">
+        <is>
+          <t>10-reconciliation-ledger.md</t>
+        </is>
+      </c>
+      <c r="N16" s="6" t="inlineStr">
+        <is>
+          <t>2026-07-01</t>
+        </is>
+      </c>
+      <c r="O16" s="6" t="inlineStr">
+        <is>
+          <t>NOT leadership headline metric</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="6" t="inlineStr">
+        <is>
+          <t>Legacy Unite</t>
+        </is>
+      </c>
+      <c r="B17" s="6" t="inlineStr">
+        <is>
+          <t>High-priority member portal</t>
+        </is>
+      </c>
+      <c r="C17" s="6" t="inlineStr">
+        <is>
+          <t>Daily nightly modules</t>
+        </is>
+      </c>
+      <c r="D17" s="6" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="E17" s="6" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="F17" s="6" t="inlineStr">
+        <is>
+          <t>active daily suite modules</t>
+        </is>
+      </c>
+      <c r="G17" s="6" t="inlineStr">
+        <is>
+          <t>Verified from repository + historical docs</t>
+        </is>
+      </c>
+      <c r="H17" s="6" t="inlineStr">
+        <is>
+          <t>Majority of high-priority journeys automated</t>
+        </is>
+      </c>
+      <c r="I17" s="6" t="inlineStr">
+        <is>
+          <t>Jenkins nightly referenced — live run not re-verified</t>
+        </is>
+      </c>
+      <c r="J17" s="6" t="inlineStr">
+        <is>
+          <t>STAGE1-Daily-Unite-Prime-Regression (docs)</t>
+        </is>
+      </c>
+      <c r="K17" s="6" t="inlineStr">
+        <is>
+          <t>Substantial automation for core member journeys; recurring Jenkins regression referenced in platform docs</t>
+        </is>
+      </c>
+      <c r="L17" s="6" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="M17" s="6" t="inlineStr">
+        <is>
+          <t>AM_Regression_Reports/docs/v2/00-v2-regression-overview.md</t>
+        </is>
+      </c>
+      <c r="N17" s="6" t="inlineStr">
+        <is>
+          <t>2026-07-21</t>
+        </is>
+      </c>
+      <c r="O17" s="6" t="inlineStr">
+        <is>
+          <t>~95% core flows claim is historical doc estimate — not verified denominator</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="6" t="inlineStr">
+        <is>
+          <t>Legacy Unite</t>
+        </is>
+      </c>
+      <c r="B18" s="6" t="inlineStr">
+        <is>
+          <t>High-priority member portal</t>
+        </is>
+      </c>
+      <c r="C18" s="6" t="inlineStr">
+        <is>
+          <t>Daily test methods (approx)</t>
+        </is>
+      </c>
+      <c r="D18" s="6" t="inlineStr">
+        <is>
+          <t>454</t>
+        </is>
+      </c>
+      <c r="E18" s="6" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="F18" s="6" t="inlineStr">
+        <is>
+          <t>TestNG/Cucumber methods</t>
+        </is>
+      </c>
+      <c r="G18" s="6" t="inlineStr">
+        <is>
+          <t>Historical estimate</t>
+        </is>
+      </c>
+      <c r="H18" s="6" t="inlineStr">
+        <is>
+          <t>10 modules with automation</t>
+        </is>
+      </c>
+      <c r="I18" s="6" t="inlineStr">
+        <is>
+          <t>Referenced nightly</t>
+        </is>
+      </c>
+      <c r="J18" s="6" t="inlineStr">
+        <is>
+          <t>See Jenkins docs</t>
+        </is>
+      </c>
+      <c r="K18" s="6" t="inlineStr">
+        <is>
+          <t>Enrollment contributions withdrawals balance login registration UGift investment options covered in daily modules</t>
+        </is>
+      </c>
+      <c r="L18" s="6" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="M18" s="6" t="inlineStr">
+        <is>
+          <t>v2/00-v2-regression-overview.md</t>
+        </is>
+      </c>
+      <c r="N18" s="6" t="inlineStr">
+        <is>
+          <t>2026-07-21</t>
+        </is>
+      </c>
+      <c r="O18" s="6" t="inlineStr"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="6" t="inlineStr">
+        <is>
+          <t>Legacy Unite</t>
+        </is>
+      </c>
+      <c r="B19" s="6" t="inlineStr">
+        <is>
+          <t>Full V2 repository</t>
+        </is>
+      </c>
+      <c r="C19" s="6" t="inlineStr">
+        <is>
+          <t>Feature files</t>
+        </is>
+      </c>
+      <c r="D19" s="6" t="inlineStr">
+        <is>
+          <t>1538</t>
+        </is>
+      </c>
+      <c r="E19" s="6" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="F19" s="6" t="inlineStr">
+        <is>
+          <t>Cucumber feature files</t>
+        </is>
+      </c>
+      <c r="G19" s="6" t="inlineStr">
+        <is>
+          <t>Verified from repository code</t>
+        </is>
+      </c>
+      <c r="H19" s="6" t="inlineStr">
+        <is>
+          <t>Extensive code assets</t>
+        </is>
+      </c>
+      <c r="I19" s="6" t="inlineStr">
+        <is>
+          <t>Execution varies by suite</t>
+        </is>
+      </c>
+      <c r="J19" s="6" t="inlineStr">
+        <is>
+          <t>Not on GitLab V3 schedule</t>
+        </is>
+      </c>
+      <c r="K19" s="6" t="inlineStr">
+        <is>
+          <t>Extensive existing automation requiring revalidation and governed suite activation</t>
+        </is>
+      </c>
+      <c r="L19" s="6" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="M19" s="6" t="inlineStr">
+        <is>
+          <t>unite-test-automation feature scan</t>
+        </is>
+      </c>
+      <c r="N19" s="6" t="inlineStr">
+        <is>
+          <t>2026-07-21</t>
+        </is>
+      </c>
+      <c r="O19" s="6" t="inlineStr"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="6" t="inlineStr">
+        <is>
+          <t>Legacy Unite</t>
+        </is>
+      </c>
+      <c r="B20" s="6" t="inlineStr">
+        <is>
+          <t>UP-scoped qTest inventory (technical)</t>
+        </is>
+      </c>
+      <c r="C20" s="6" t="inlineStr">
+        <is>
+          <t>Executed qTest cases</t>
+        </is>
+      </c>
+      <c r="D20" s="6" t="inlineStr">
+        <is>
+          <t>268</t>
+        </is>
+      </c>
+      <c r="E20" s="6" t="inlineStr">
+        <is>
+          <t>744</t>
+        </is>
+      </c>
+      <c r="F20" s="6" t="inlineStr">
+        <is>
+          <t>qTest cases</t>
+        </is>
+      </c>
+      <c r="G20" s="6" t="inlineStr">
+        <is>
+          <t>Verified inventory share only — stale</t>
+        </is>
+      </c>
+      <c r="H20" s="6" t="inlineStr">
+        <is>
+          <t>Mapped cases exist</t>
+        </is>
+      </c>
+      <c r="I20" s="6" t="inlineStr">
+        <is>
+          <t>Stale export 2026-06-29</t>
+        </is>
+      </c>
+      <c r="J20" s="6" t="inlineStr">
+        <is>
+          <t>Jenkins/Ant legacy</t>
+        </is>
+      </c>
+      <c r="K20" s="6" t="inlineStr">
+        <is>
+          <t>Technical appendix only — not functional completeness</t>
+        </is>
+      </c>
+      <c r="L20" s="6" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="M20" s="6" t="inlineStr">
+        <is>
+          <t>10-reconciliation-ledger.md</t>
+        </is>
+      </c>
+      <c r="N20" s="6" t="inlineStr">
+        <is>
+          <t>2026-06-29</t>
+        </is>
+      </c>
+      <c r="O20" s="6" t="inlineStr">
+        <is>
+          <t>NOT leadership headline metric</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="6" t="inlineStr">
+        <is>
+          <t>Legacy Unite</t>
+        </is>
+      </c>
+      <c r="B21" s="6" t="inlineStr">
+        <is>
+          <t>CSR / management / green screens</t>
+        </is>
+      </c>
+      <c r="C21" s="6" t="inlineStr">
+        <is>
+          <t>CSR maintenance + greenscreen features</t>
+        </is>
+      </c>
+      <c r="D21" s="6" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="E21" s="6" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="F21" s="6" t="inlineStr">
+        <is>
+          <t>feature scenarios</t>
+        </is>
+      </c>
+      <c r="G21" s="6" t="inlineStr">
+        <is>
+          <t>Program estimate requiring reconciliation</t>
+        </is>
+      </c>
+      <c r="H21" s="6" t="inlineStr">
+        <is>
+          <t>Automation assets exist</t>
+        </is>
+      </c>
+      <c r="I21" s="6" t="inlineStr">
+        <is>
+          <t>Not in 10 daily modules</t>
+        </is>
+      </c>
+      <c r="J21" s="6" t="inlineStr">
+        <is>
+          <t>Manual / deferred suites</t>
+        </is>
+      </c>
+      <c r="K21" s="6" t="inlineStr">
+        <is>
+          <t>Automation assets exist but require revalidation synchronization and inclusion in governed nightly suite</t>
+        </is>
+      </c>
+      <c r="L21" s="6" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="M21" s="6" t="inlineStr">
+        <is>
+          <t>unite/testsuite/csr/</t>
+        </is>
+      </c>
+      <c r="N21" s="6" t="inlineStr">
+        <is>
+          <t>2026-07-21</t>
+        </is>
+      </c>
+      <c r="O21" s="6" t="inlineStr"/>
+    </row>
+    <row r="22">
+      <c r="A22" s="6" t="inlineStr">
+        <is>
+          <t>Back-office / Batch</t>
+        </is>
+      </c>
+      <c r="B22" s="6" t="inlineStr">
+        <is>
+          <t>Backoffice subtree</t>
+        </is>
+      </c>
+      <c r="C22" s="6" t="inlineStr">
+        <is>
+          <t>Feature files</t>
+        </is>
+      </c>
+      <c r="D22" s="6" t="inlineStr">
+        <is>
+          <t>1062</t>
+        </is>
+      </c>
+      <c r="E22" s="6" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="F22" s="6" t="inlineStr">
+        <is>
+          <t>Cucumber features</t>
+        </is>
+      </c>
+      <c r="G22" s="6" t="inlineStr">
+        <is>
+          <t>Verified from repository code</t>
+        </is>
+      </c>
+      <c r="H22" s="6" t="inlineStr">
+        <is>
+          <t>Substantial implementation</t>
+        </is>
+      </c>
+      <c r="I22" s="6" t="inlineStr">
+        <is>
+          <t>Weekly backoffice referenced Tue/Wed</t>
+        </is>
+      </c>
+      <c r="J22" s="6" t="inlineStr">
+        <is>
+          <t>Not on V3 GitLab nightly</t>
+        </is>
+      </c>
+      <c r="K22" s="6" t="inlineStr">
+        <is>
+          <t>Back-office automation implemented; recurring inclusion requires revalidation and schedule confirmation</t>
+        </is>
+      </c>
+      <c r="L22" s="6" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="M22" s="6" t="inlineStr">
+        <is>
+          <t>unite/testsuite/backoffice/</t>
+        </is>
+      </c>
+      <c r="N22" s="6" t="inlineStr">
+        <is>
+          <t>2026-07-21</t>
+        </is>
+      </c>
+      <c r="O22" s="6" t="inlineStr">
+        <is>
+          <t>Kofax/feed flows in backoffice tree</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="6" t="inlineStr">
+        <is>
+          <t>ASTRO / SFRP</t>
+        </is>
+      </c>
+      <c r="B23" s="6" t="inlineStr">
+        <is>
+          <t>ASTRO UI</t>
+        </is>
+      </c>
+      <c r="C23" s="6" t="inlineStr">
+        <is>
+          <t>Feature files</t>
+        </is>
+      </c>
+      <c r="D23" s="6" t="inlineStr">
+        <is>
+          <t>391</t>
+        </is>
+      </c>
+      <c r="E23" s="6" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="F23" s="6" t="inlineStr">
+        <is>
+          <t>Cucumber features</t>
+        </is>
+      </c>
+      <c r="G23" s="6" t="inlineStr">
+        <is>
+          <t>Verified from repository code</t>
+        </is>
+      </c>
+      <c r="H23" s="6" t="inlineStr">
+        <is>
+          <t>Substantial asset base</t>
+        </is>
+      </c>
+      <c r="I23" s="6" t="inlineStr">
+        <is>
+          <t>No verified recurring execution</t>
+        </is>
+      </c>
+      <c r="J23" s="6" t="inlineStr">
+        <is>
+          <t>ASTRO-TB-REFRESH prep only</t>
+        </is>
+      </c>
+      <c r="K23" s="6" t="inlineStr">
+        <is>
+          <t>ASTRO has substantial existing automation assets; recurring execution inactive — suites require revalidation before active regression coverage</t>
+        </is>
+      </c>
+      <c r="L23" s="6" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="M23" s="6" t="inlineStr">
+        <is>
+          <t>astro-test-automation feature scan</t>
+        </is>
+      </c>
+      <c r="N23" s="6" t="inlineStr">
+        <is>
+          <t>2026-07-21</t>
+        </is>
+      </c>
+      <c r="O23" s="6" t="inlineStr">
+        <is>
+          <t>1236 scenario count from prior scan — use features as stable unit</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="6" t="inlineStr">
+        <is>
+          <t>ASTRO / SFRP</t>
+        </is>
+      </c>
+      <c r="B24" s="6" t="inlineStr">
+        <is>
+          <t>ASTRO API</t>
+        </is>
+      </c>
+      <c r="C24" s="6" t="inlineStr">
+        <is>
+          <t>Test classes</t>
+        </is>
+      </c>
+      <c r="D24" s="6" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="E24" s="6" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="F24" s="6" t="inlineStr">
+        <is>
+          <t>API test classes</t>
+        </is>
+      </c>
+      <c r="G24" s="6" t="inlineStr">
+        <is>
+          <t>Verified implementation estimate</t>
+        </is>
+      </c>
+      <c r="H24" s="6" t="inlineStr">
+        <is>
+          <t>Small API module</t>
+        </is>
+      </c>
+      <c r="I24" s="6" t="inlineStr">
+        <is>
+          <t>No schedule</t>
+        </is>
+      </c>
+      <c r="J24" s="6" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="K24" s="6" t="inlineStr">
+        <is>
+          <t>API automation footprint small; scope vs GS priority TBD</t>
+        </is>
+      </c>
+      <c r="L24" s="6" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="M24" s="6" t="inlineStr">
+        <is>
+          <t>api-test-automation/astro/</t>
+        </is>
+      </c>
+      <c r="N24" s="6" t="inlineStr">
+        <is>
+          <t>2026-07-21</t>
+        </is>
+      </c>
+      <c r="O24" s="6" t="inlineStr"/>
+    </row>
+    <row r="25">
+      <c r="A25" s="6" t="inlineStr">
+        <is>
+          <t>COPACS</t>
+        </is>
+      </c>
+      <c r="B25" s="6" t="inlineStr">
+        <is>
+          <t>Platform scope</t>
+        </is>
+      </c>
+      <c r="C25" s="6" t="inlineStr">
+        <is>
+          <t>Automation identified</t>
+        </is>
+      </c>
+      <c r="D25" s="6" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E25" s="6" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="F25" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="G25" s="6" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="H25" s="6" t="inlineStr">
+        <is>
+          <t>No validated automation in reviewed repos</t>
+        </is>
+      </c>
+      <c r="I25" s="6" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="J25" s="6" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="K25" s="6" t="inlineStr">
+        <is>
+          <t>Scope and ownership require business discovery</t>
+        </is>
+      </c>
+      <c r="L25" s="6" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="M25" s="6" t="inlineStr">
+        <is>
+          <t>leadership-decision-log D-10</t>
+        </is>
+      </c>
+      <c r="N25" s="6" t="inlineStr">
+        <is>
+          <t>2026-07-21</t>
+        </is>
+      </c>
+      <c r="O25" s="6" t="inlineStr"/>
+    </row>
+    <row r="26">
+      <c r="A26" s="6" t="inlineStr">
+        <is>
+          <t>Performance</t>
+        </is>
+      </c>
+      <c r="B26" s="6" t="inlineStr">
+        <is>
+          <t>IDP</t>
+        </is>
+      </c>
+      <c r="C26" s="6" t="inlineStr">
+        <is>
+          <t>Scheduled perf suite</t>
+        </is>
+      </c>
+      <c r="D26" s="6" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="E26" s="6" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="F26" s="6" t="inlineStr">
+        <is>
+          <t>perf regression job</t>
+        </is>
+      </c>
+      <c r="G26" s="6" t="inlineStr">
+        <is>
+          <t>Verified from KB evidence</t>
+        </is>
+      </c>
+      <c r="H26" s="6" t="inlineStr">
+        <is>
+          <t>Scripts exist</t>
+        </is>
+      </c>
+      <c r="I26" s="6" t="inlineStr">
+        <is>
+          <t>Referenced weekdays ~3 AM</t>
+        </is>
+      </c>
+      <c r="J26" s="6" t="inlineStr">
+        <is>
+          <t>AGSUP_IDP_REGRESSION_SUITE</t>
+        </is>
+      </c>
+      <c r="K26" s="6" t="inlineStr">
+        <is>
+          <t>IDP performance regression on schedule; functional gate separate</t>
+        </is>
+      </c>
+      <c r="L26" s="6" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="M26" s="6" t="inlineStr">
+        <is>
+          <t>perf tracker 2026-07-02</t>
+        </is>
+      </c>
+      <c r="N26" s="6" t="inlineStr">
+        <is>
+          <t>2026-07-02</t>
+        </is>
+      </c>
+      <c r="O26" s="6" t="inlineStr"/>
+    </row>
+    <row r="27">
+      <c r="A27" s="6" t="inlineStr">
+        <is>
+          <t>Performance</t>
+        </is>
+      </c>
+      <c r="B27" s="6" t="inlineStr">
+        <is>
+          <t>MSC Mobile</t>
+        </is>
+      </c>
+      <c r="C27" s="6" t="inlineStr">
+        <is>
+          <t>Perf scripts</t>
+        </is>
+      </c>
+      <c r="D27" s="6" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="E27" s="6" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="F27" s="6" t="inlineStr">
+        <is>
+          <t>JMX/YAML pairs</t>
+        </is>
+      </c>
+      <c r="G27" s="6" t="inlineStr">
+        <is>
+          <t>Verified manually executable</t>
+        </is>
+      </c>
+      <c r="H27" s="6" t="inlineStr">
+        <is>
+          <t>Scripts exist</t>
+        </is>
+      </c>
+      <c r="I27" s="6" t="inlineStr">
+        <is>
+          <t>Manual only</t>
+        </is>
+      </c>
+      <c r="J27" s="6" t="inlineStr">
+        <is>
+          <t>AGSUP_UNITE_MSC_ENDURANCE manual</t>
+        </is>
+      </c>
+      <c r="K27" s="6" t="inlineStr">
+        <is>
+          <t>MSC performance scripts exist; no periodic trigger confirmed</t>
+        </is>
+      </c>
+      <c r="L27" s="6" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="M27" s="6" t="inlineStr">
+        <is>
+          <t>performance/mobile/unite-msc/</t>
+        </is>
+      </c>
+      <c r="N27" s="6" t="inlineStr">
+        <is>
+          <t>2026-07-02</t>
+        </is>
+      </c>
+      <c r="O27" s="6" t="inlineStr"/>
+    </row>
+    <row r="28">
+      <c r="A28" s="6" t="inlineStr">
+        <is>
+          <t>Reporting / Governance</t>
+        </is>
+      </c>
+      <c r="B28" s="6" t="inlineStr">
+        <is>
+          <t>qTest manual inventory</t>
+        </is>
+      </c>
+      <c r="C28" s="6" t="inlineStr">
+        <is>
+          <t>Executed cases (V2 export)</t>
+        </is>
+      </c>
+      <c r="D28" s="6" t="inlineStr">
+        <is>
+          <t>744</t>
+        </is>
+      </c>
+      <c r="E28" s="6" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="F28" s="6" t="inlineStr">
+        <is>
+          <t>qTest cases</t>
+        </is>
+      </c>
+      <c r="G28" s="6" t="inlineStr">
+        <is>
+          <t>Stale execution evidence</t>
+        </is>
+      </c>
+      <c r="H28" s="6" t="inlineStr">
+        <is>
+          <t>Inventory exists</t>
+        </is>
+      </c>
+      <c r="I28" s="6" t="inlineStr">
+        <is>
+          <t>2026-06-29 snapshot</t>
+        </is>
+      </c>
+      <c r="J28" s="6" t="inlineStr">
+        <is>
+          <t>No live API</t>
+        </is>
+      </c>
+      <c r="K28" s="6" t="inlineStr">
+        <is>
+          <t>qTest data stale; row-level IDs not exported</t>
+        </is>
+      </c>
+      <c r="L28" s="6" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="M28" s="6" t="inlineStr">
+        <is>
+          <t>v2-qtest-jenkins export</t>
+        </is>
+      </c>
+      <c r="N28" s="6" t="inlineStr">
+        <is>
+          <t>2026-06-29</t>
+        </is>
+      </c>
+      <c r="O28" s="6" t="inlineStr"/>
+    </row>
+    <row r="29">
+      <c r="A29" s="6" t="inlineStr">
+        <is>
+          <t>Reporting / Governance</t>
+        </is>
+      </c>
+      <c r="B29" s="6" t="inlineStr">
+        <is>
+          <t>Coverage register</t>
+        </is>
+      </c>
+      <c r="C29" s="6" t="inlineStr">
+        <is>
+          <t>Platform metrics with status labels</t>
+        </is>
+      </c>
+      <c r="D29" s="6" t="inlineStr">
+        <is>
+          <t>11</t>
+        </is>
+      </c>
+      <c r="E29" s="6" t="inlineStr">
+        <is>
+          <t>11</t>
+        </is>
+      </c>
+      <c r="F29" s="6" t="inlineStr">
+        <is>
+          <t>register rows</t>
+        </is>
+      </c>
+      <c r="G29" s="6" t="inlineStr">
+        <is>
+          <t>Verified</t>
+        </is>
+      </c>
+      <c r="H29" s="6" t="inlineStr">
+        <is>
+          <t>Register maintained</t>
+        </is>
+      </c>
+      <c r="I29" s="6" t="inlineStr">
+        <is>
+          <t>Partial live collectors</t>
+        </is>
+      </c>
+      <c r="J29" s="6" t="inlineStr">
+        <is>
+          <t>Partial</t>
+        </is>
+      </c>
+      <c r="K29" s="6" t="inlineStr">
+        <is>
+          <t>Automated harmonized register feasible; APIs blocked</t>
+        </is>
+      </c>
+      <c r="L29" s="6" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="M29" s="6" t="inlineStr">
+        <is>
+          <t>verified-metrics-register.csv</t>
+        </is>
+      </c>
+      <c r="N29" s="6" t="inlineStr">
+        <is>
+          <t>2026-07-21</t>
+        </is>
+      </c>
+      <c r="O29" s="6" t="inlineStr"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:U21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -973,10 +3162,10 @@
     <col width="41" customWidth="1" min="7" max="7"/>
     <col width="48" customWidth="1" min="8" max="8"/>
     <col width="36" customWidth="1" min="9" max="9"/>
-    <col width="36" customWidth="1" min="10" max="10"/>
+    <col width="44" customWidth="1" min="10" max="10"/>
     <col width="48" customWidth="1" min="11" max="11"/>
     <col width="48" customWidth="1" min="12" max="12"/>
-    <col width="48" customWidth="1" min="13" max="13"/>
+    <col width="40" customWidth="1" min="13" max="13"/>
     <col width="48" customWidth="1" min="14" max="14"/>
     <col width="48" customWidth="1" min="15" max="15"/>
     <col width="36" customWidth="1" min="16" max="16"/>
@@ -1769,7 +3958,7 @@
       </c>
       <c r="G8" s="6" t="inlineStr">
         <is>
-          <t>22 verified L3+ endpoints</t>
+          <t>24 implemented L3+ endpoints</t>
         </is>
       </c>
       <c r="H8" s="6" t="inlineStr">
@@ -1779,17 +3968,17 @@
       </c>
       <c r="I8" s="6" t="inlineStr">
         <is>
-          <t>22</t>
+          <t>24</t>
         </is>
       </c>
       <c r="J8" s="6" t="inlineStr">
         <is>
-          <t>88.0% verified endpoint automation</t>
+          <t>96.0% implemented automation</t>
         </is>
       </c>
       <c r="K8" s="6" t="inlineStr">
         <is>
-          <t>Verified sign-off 2026-07-14; projected 24/25 (96%) pending QC4+Stage1 rerun</t>
+          <t>Verified in code @ cee0de9; 88% stale execution @ 7ccaf46</t>
         </is>
       </c>
       <c r="L8" s="6" t="inlineStr">
@@ -1799,7 +3988,7 @@
       </c>
       <c r="M8" s="6" t="inlineStr">
         <is>
-          <t>GHA Dashboard slice validated external; module expansion in progress</t>
+          <t>GHA Dashboard slice validated external</t>
         </is>
       </c>
       <c r="N8" s="6" t="inlineStr">
@@ -1824,7 +4013,7 @@
       </c>
       <c r="R8" s="6" t="inlineStr">
         <is>
-          <t>17-mobile2-api-automation-signoff.md @ 7ccaf46; code @ cee0de9</t>
+          <t>mobile2-endpoint-current-state.csv @ cee0de9</t>
         </is>
       </c>
       <c r="S8" s="6" t="inlineStr">
@@ -1834,12 +4023,12 @@
       </c>
       <c r="T8" s="6" t="inlineStr">
         <is>
-          <t>Verified baseline — sign-off path open</t>
+          <t>Implemented — execution refresh pending</t>
         </is>
       </c>
       <c r="U8" s="6" t="inlineStr">
         <is>
-          <t>YTD + GET mobilebanks/{id} in code pending evidence; mobilemembers excluded from automation numerator; QA-1405 nightly</t>
+          <t>mobilemembers excluded from numerator; destructive ops smoke/module only; QA-1405 nightly</t>
         </is>
       </c>
     </row>
@@ -1876,7 +4065,7 @@
       </c>
       <c r="G9" s="6" t="inlineStr">
         <is>
-          <t>1 verified + 5 implemented pending</t>
+          <t>6 implemented endpoint identities</t>
         </is>
       </c>
       <c r="H9" s="6" t="inlineStr">
@@ -1886,17 +4075,17 @@
       </c>
       <c r="I9" s="6" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>6</t>
         </is>
       </c>
       <c r="J9" s="6" t="inlineStr">
         <is>
-          <t>3.7% verified (1/27)</t>
+          <t>22.2% implemented; 3.7% execution-verified</t>
         </is>
       </c>
       <c r="K9" s="6" t="inlineStr">
         <is>
-          <t>Verified session; 5 endpoints implemented pending evidence</t>
+          <t>6 in code @ cee0de9; 1 execution-verified session</t>
         </is>
       </c>
       <c r="L9" s="6" t="inlineStr">
@@ -1921,7 +4110,7 @@
       </c>
       <c r="P9" s="6" t="inlineStr">
         <is>
-          <t>okdirect + nmdirect (auth)</t>
+          <t>okdirect + nmdirect</t>
         </is>
       </c>
       <c r="Q9" s="6" t="inlineStr">
@@ -1931,7 +4120,7 @@
       </c>
       <c r="R9" s="6" t="inlineStr">
         <is>
-          <t>03-document-postman-coverage-matrix.md; mobile/mobile1 @ cee0de9</t>
+          <t>mobile1-endpoint-current-state.csv @ cee0de9</t>
         </is>
       </c>
       <c r="S9" s="6" t="inlineStr">
@@ -1946,7 +4135,7 @@
       </c>
       <c r="U9" s="6" t="inlineStr">
         <is>
-          <t>Leadership baseline 1/27; potential 6/27 after workbook mapping + execution evidence</t>
+          <t>21 endpoints remain; 5 new endpoints need execution evidence</t>
         </is>
       </c>
     </row>
@@ -3240,7 +5429,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -4482,7 +6671,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>

</xml_diff>